<commit_message>
feat: publish latest complete project snapshot
</commit_message>
<xml_diff>
--- a/data-service/data/参阅信息.xlsx
+++ b/data-service/data/参阅信息.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\project\icbc\data-service\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44957262-2445-4988-A634-7D96E60605D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5FB576B5-427B-4042-8D08-AB1BC1B865D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="12600" yWindow="870" windowWidth="15315" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,16 +58,10 @@
     <t>&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;国内外重要行业动态&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据新华财经报道，在6月16日开幕的2026中国国际金融展上，数字人民币国际运营中心与首批26家金融机构在沪签署直接参与者服务协议，“数币达”（简称 CBETS）跨境结算综合服务平台参与者可依托CBETS的系统能力为客户提供低成本、多元化和安全高效的跨境数字支付服务。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据新华财经报道，欧洲议会16日批准落实与美国达成的关税协议。此前欧盟成员国已批准该协议，这意味着欧洲议会议员的批准成为协议实施前最后一个政治步骤，使欧盟有望按时赶在美国总统特朗普设定的7月4日期限前完成程序，以化解美方加征关税的威胁。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;转型社会的“独有所托”治理&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;如今，人口老龄化步步加深、传统大家庭慢慢“解体”、人口跨城流动成为常态，“独自生活”早已不是小众现象。对应的“独有所托”，也不再是简单的民生小事，而是关乎社会稳定、治理水平和城市文明温度的核心社会考题。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;很多人对“独”的印象，还停留在古时候“鳏寡孤独、无人依靠”的狭义认知，但放在今天，这个字的内涵早已全面升级。它不再单指无依无靠的老人，而是囊括了独居老人、独居青年、失独家庭、无亲属照料的残疾人等一大类多元群体。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;这种全新的“独居形态”，正在给我们的社会治理体系抛出全新挑战，也倒逼传统的帮扶模式必须更新迭代、跟上时代节奏。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;其实我国帮扶特殊独居群体，有着源远流长的“仁政传统”。从先秦《周礼》“保息六养万民”、管仲“九惠之教”，到唐宋元明清的官办救助机构与常态化赈济，形成了以“仁政”为核心、“亲属优先+政府兜底”为格局、物质帮扶为重点的传统模式。这一模式契合了古代社会生产力水平与治理需求，但在当代社会转型背景下，已完全难以适配“独”的新变化、新需求，“独有所托”的治理重心，必须全面转向当代群体的核心痛点与现实诉求。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;当代社会中，“独”的群体已发生质的蜕变，呈现出多元化、年轻化、规模化的鲜明特征，彻底打破了“独居是老年人专利”的固有认知，这也是当前“独有所托”治理面临的首要前提。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;数据最能说明问题：截至2024年，我国独居人口已经达到1.23亿，这是一个堪比大国总人口的庞大群体。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;这其中，既有老年独居群体：全国超3.1亿60岁以上老人里，有14.2%是独居状态。他们大多因为子女异地打拼、亲属分散疏离，独自面对岁月带来的难题，一旦遭遇失能失智、突发疾病，常常陷入“身边无人、求助无门”的窘迫困境。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;更让人意外的是，年轻独居群体早已成为主力军。因为读书年限变长、结婚生育推迟、职业跨城流动、生活观念更加独立，越来越多年轻人主动选择独居生活。他们或许经济独立、衣食无忧，却躲不开新时代的独居痛点：常年独处的孤独感、突发意外无人帮忙、心理压力无处疏导，看似自由的独居生活，藏着不少隐形风险。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;除此之外，失独家庭、无亲属照料的残疾人等群体，彻底失去了家庭支撑，常年面临监护缺位、权益没人保障的现实难题。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;贝壳研究院更是预测，2030年我国独居人口规模将突破至2亿。足以可见，独居已经成为不可逆的社会新常态，治理模式如果还守着老一套，注定行不通，必须精准适配新变化、新需求。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;群体变了，但治理服务的更新速度没能及时跟上，这就导致了明显的“制度脱节”和“服务缺口”，原本只是个体的独居困境，慢慢演变成了系统性的社会问题。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;2025年《中华遗嘱库白皮书》的数据很直观：立遗嘱的人群中，空巢老人占比高达61%，孤寡老人占5.09%。曾经最可靠的家庭监护模式，在人口流动、亲属疏离的当下，正在慢慢弱化甚至断裂。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;现实中的扎心案例比比皆是：独居老人突发重病，因为没有亲属在场签字，耽误最佳救治时机；老人失能失智后，无人照料、无人看护；独居青年深夜遇到意外，求助无门；无亲属照料的特殊群体，名下财产没人打理、身后事务无人处置……&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;前段时间46岁独身蒋女士的经历，就是最真实的缩影：突发脑出血昏迷，因无人签字导致医疗决策受阻，不幸离世后，数百万元资产陷入处置僵局。这一桩个案，精准戳中了当代独居群体“有收入、有生活、却无依靠”的监护短板，也足以说明，针对新型独居群体搭建专属治理体系，已经迫在眉睫。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;面对独居群体的新特征、治理工作的新困境，我们必须跳出传统“送米送油、给钱给物”的单一救助思维。不再只聚焦“活下去”的生存保障，更要追求“活得好、有尊严”的品质保障；不再是等困难发生后被动救助，而是主动前置服务、赋能个体，搭建一套适配新时代的系统化保障体系。具体可以参考四个维度：&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;一是最基本的。聚焦“监护缺位”痛点，强化制度兜底，破解当代“独”类群体的核心困境。针对当代独居群体亲属支撑薄弱、监护责任缺失的问题，加快“独有所托”专项立法进程，明确独居群体的界定、权利保障、救助标准与责任分工，重点强化意定监护制度的普及与落实。同时，完善医疗急救、财产管理、身后事务处置等配套制度，破解“无人签字”“财产冻结”“身后事无人料理”等痛点。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;二是需注意的。立足“群体多元”特征，分类精准施策，适配不同独居群体的差异化需求。当代“独”的群体构成复杂，需求差异显著，需摒弃“一刀切”的救助模式，实现精准滴灌。针对独居老人，重点强化居家照护、医疗保障与应急响应；针对独居青年，聚焦应急处置、心理疏导与生活赋能；针对失独家庭、无亲属照料的残疾人，重点强化生活照料、精神慰藉与权利保障。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;三是可依托的。激活“协同治理”动能，构建多元体系，强化当代“独”类群体的支撑网络。打破“政府单一兜底”的传统模式，构建“政府主导、家庭补充、社区联动、社会参与”的协同治理格局。一方面，强化家庭补充作用，对照料独居老人、独居残疾人的亲属给予补贴、税收减免等优惠政策，减轻照料负担，激发家庭照料的积极性；另一方面，激活基层与社会力量，依托社区建立独居群体档案，组织邻里、志愿者提供物资代购、临时照料等服务；同时，引导社会组织、专业机构参与，提供专业监护、心理疏导、技能培训等服务，形成全方位、多层次的支撑网络。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;四是最重要的。强化“内生赋能”导向，提升自我保障能力，实现“独有所托”的长效发展。最好的保障，不止是外界帮扶，更是让独居人群拥有自我保障、独立生活的能力。美国、加拿大“独居者互助小组”模式，通过组织独居者相互帮扶、交流经验，既提升自我保障能力，也缓解独居带来的孤独感，实现“被动帮扶”向“主动自救”的转变。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;最终分析结论（Final Analysis Conclusion）：&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;社会转型带来“独”的群体新变化，也催生“独有所托”的治理新命题。传统治理模式为我们提供了“以人为本”的价值底色，但唯有把握“独”的新形态、新需求，才有可能有效破解当代“独有所托”的治理困境，让每一个独居群体都能获得有尊严、有保障的生活。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;5月社零转负反映国内消费市场疲软&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;国家统计局数据显示，2026年5月社会消费品零售总额同比下降0.6%，为2023年以来首次转负；剔除汽车后的消费品零售额同比增长1.1%，较上月进一步回落。从环比看，5月社零总额下降0.38%，已连续三个月负增长，表明春节后消费恢复动能持续减弱。与此同时，1—5月服务零售额同比增长5.4%，明显高于商品零售增速，消费结构分化进一步扩大。从具体领域看，商品零售已连续两个月下降。此前受“以旧换新”政策刺激的耐用消费品普遍回落，家电和音响器材类消费同比下降15.6%，汽车类消费下降16.1%，新能源汽车购置税优惠退坡以及前期需求透支效应持续显现。国际金价回调导致金银珠宝消费继续负增长，房地产市场低迷则拖累建筑装潢材料消费。相比之下，粮油食品、服装鞋帽等基本生活类消费仍保持增长，但难以弥补大宗消费品下滑带来的影响。从长期趋势看，目前消费增速已明显低于正常年份水平。过去较长时期内，中国消费增长虽然不是经济增长的主要驱动力，但社会消费品零售总额通常能够维持4%左右甚至更高的增长水平，波动相对有限。如今社零首次转负，说明居民消费能力和消费意愿仍未完全恢复，房地产调整、收入预期偏弱以及耐用品需求提前释放等因素正在共同作用。展望未来，若就业、收入和资产价格预期难以改善，仅依靠阶段性补贴政策恐难持续支撑消费增长，居民消费信心修复仍将是扩大内需的关键所在。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;部分中下游企业面临阶段性成本压力&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;国家统计局国民经济综合统计司副司长王冠华表示，目前尽管PPI涨幅扩大，但是CPI运行总体平稳。这其中原因主要有以下几点：首先，PPI向CPI的传导主要集中在工业消费品领域，而在CPI当中占比较大的食品价格和服务价格受工业品价格波动影响较小。第二，上游的工业品价格受国际大宗商品价格影响较为直接，但沿着产业链条向中下游传导到居民终端消费市场，这个过程会受到市场竞争、技术进步等因素影响，往往呈现沿着产业链递减特点。第三，我国经济运行总体平稳，产业链供应链韧性较强，商品和服务供给比较充裕，各项保供稳价政策有力有效。王冠华表示，关于成本上升给企业带来的经营压力，这个问题确实需要关注。受产业链分工不同，市场需求、行业竞争等多重因素影响，行业之间盈利表现呈现一定分化，部分中下游企业面临阶段性成本压力。面对成本变化，很多企业主动作为，通过技术改造、精细化管理、拓展市场等方式挖潜增效、对冲压力；相关部门和地区持续落实落细助企政策，支持企业大规模设备更新改造，采取措施降低企业用能、物流等成本，效果有望逐步显现。从全国层面来看，尽管部分企业生产经营仍有压力，但随着工业生产较快增长，工业品价格回升，工业企业营业收入和利润保持了稳步增长，工业经济的韧性继续显现。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;战略性矿产全面进入“国家统管”新阶段&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;我国战略性矿产全面迈入“国家统管”新阶段。日前，《中华人民共和国矿产资源法实施条例》正式实施，稀土、钨、锂、钴、镓、锗等36种关键矿产被列入国家级战略性矿产资源目录。这标志着我国战略性矿产管理由分散监管转向“探产供储销”全链条统筹，关键矿产供给、储备和产业运行逻辑将迎来系统性调整。在顶层设计上，《条例》明确，国家将在财政、金融、土地、生态环境、产业、进出口等方面完善支持政策，加大战略性矿产勘查、开采、加工、贸易和储备力度，提升矿产资源安全保障水平。对特定战略性矿产，还将实行规划管控、总量调控和限定开采主体等保护性措施。供给端方面，《条例》进一步完善矿业权设立方式，明确优先通过招标出让以及可协议出让的具体情形。对于保障国家矿产资源安全急需开采的战略性矿产，经国务院同意，可直接授予采矿权。在市场运行层面，《条例》强化产能储备和国家储备安排，从市场定价转向战略定价。战略性矿产采矿权人需结合生产能力、运输条件和安全状况等编制产能储备建设方案，确保应急增产能力；纳入产地储备的资源原则上储备期不少于五年，未经批准不得开采或压覆。业内认为，新规有助于遏制上游无序扩张，并根据新能源、高端制造等下游需求调节供给节奏，为关键矿产安全供给装上“稳定阀”。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;房市分化延续一线回暖而二三线走弱&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;6月16日，国家统计局发布5月70城住宅价格统计，市场呈现一线价格走强、二三线持续走弱的分化格局。当月一线城市新房环比涨0.2%，涨幅较4月扩大0.1个百分点，上海、广州、深圳新房小幅上行，北京新房环比回落0.2%。二线新房环比跌幅维持0.1%不变，三线新房环比跌幅扩大至0.4%，新房价格环比上涨城市共16个，较上月仅增加2个。二手房分化进一步加剧，一线二手房环比稳定上涨0.4%，上海、深圳涨幅达0.6%，二线二手房跌幅持平于0.2%，三线二手房跌幅同步扩大0.1个百分点，二手房价格上涨城市缩减至10个。人口持续向核心城市集聚、改善置换需求集中释放，支撑一线房价走出独立行情，而多数二三线城市面临人口流出、新房库存高企的双重压力，购房需求持续走弱，进而拉大各线城市价格走势差距。楼市结构性修复仅局限于一线城市核心房源，短期能够带动核心区域房产流动性改善，但难以向低能级城市传导。中长期市场风险持续存在，三线城市房价下跌幅度持续加深，库存去化周期不断拉长，地方房企回款压力将进一步抬升；二手房上涨城市数量收缩，说明存量房市场修复动能不足，当下楼市整体难以形成全面企稳行情。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;青年就业仍是下半年宏观政策的重要约束&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;中国经济当前最突出的问题并不是生产能力不足，是需求偏弱和就业承压相互强化。5月全国城镇调查失业率从4月的5.2%降至5.1%，表面看有所改善，但青年就业压力并没有真正解除。今年高校毕业生规模预计达到1270万人，同比增加48万人，再创新高，毕业季集中进入劳动力市场后，16—24岁和25—29岁青年群体的就业压力还会进一步显现。此前4月不含在校生的16—24岁失业率仍有16.3%，25—29岁失业率为7.4%，都明显高于总体失业率，说明问题不是简单的季节性波动，而是教育供给、产业岗位和企业用工能力之间存在结构性错配。更重要的是，5月社零同比下降0.6%，固定资产投资前5个月下降4.1%，房地产投资下降16.2%，这些数据都指向同一个问题：居民收入预期和企业扩张意愿偏弱，会反过来压缩新增岗位。AI和高技术制造虽然增长较快，5月高技术制造业增加值增长15.1%，但其就业吸纳能力有限，难以替代房地产、服务业和民营经济过去承担的大规模就业功能。因此，下半年宏观政策不能只盯GDP增速，更要把稳就业放在更靠前的位置，通过扩大服务消费、减轻企业成本、稳定民营部门预期和增加基层公共岗位，缓解毕业生集中就业压力。青年就业稳不住，消费信心和社会预期也很难真正修复。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;需规避各国家战略间的政策冲突问题&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;6月15日，国务院总理李强在主持“强化主体功能区战略实施，促进区域协调发展”专题学习时强调，区域协调发展战略、区域重大战略、新型城镇化战略等都是基于国土空间的重大战略，要系统梳理不同国家战略中明确的空间发展格局、区域功能和实施重点，统筹推动主体功能区战略与其他国家重大战略协同叠加。这意味着，实施主体功能区战略既要充分释放战略叠加综合效能，也要防范功能错位、政策对冲的“打架”问题。当前区域协调发展、区域重大、新型城镇化、主体功能区四大战略共同构成国土开发保护顶层框架，主体功能区战略划定城市化、农业、生态三类空间底线，是所有空间战略的基础底板，区域重大战略打造长三角、黄河流域等增长极，新型城镇化聚焦城市群人口产业集聚，区域协调发展统筹四大板块均衡发展，多重战略落地时空间范围高度交叉、主管部门各有分工，天然存在目标、政策、管控规则脱节风险。现实中部分流域、市县出现发展诉求冲突，生态功能区内盲目布局产业项目、农产品主产区过度扩张城镇建设用地、都市圈建设忽视资源环境承载约束等现象，根源在于各战略单独推进、规划标准不统一，造成资源错配、治理成本抬升。因此，要想实现良性叠加，就需系统梳理各类战略开发强度、产业准入、补偿机制等实施细则，以主体功能区划定刚性底线，其他战略在此基础上差异化配套政策。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;央企产业横向布局突出问题制约稳增长目标&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;国务院国资委近期召开专题会议研究审议《中央企业“十五五”发展规划纲要》编制工作。“十四五”以来，国资央企牢牢把握产业变革方向，筑牢实体经济根基、巩固传统产业优势、厚植新兴产业潜力，战略性新兴产业领域投资年均增速超20%、营业收入规模超12万亿元，累计布局“AI+”应用场景超1200个，有力推动关键产业爬坡过坎、升级发展，在新一代信息技术、新能源、新材料、高端装备制造等领域打造了一批万亿元级产业集群。但横向比较来看，中央企业产业布局存在战线长、分布广且高端不足、低端过剩等突出问题，一些传统产业逐步进入“增长极限”，新兴产业尚未完全形成竞争优势，实现高基数上的稳增长面临更多挑战。业界人士普遍认为，当前，新一轮科技革命和产业变革加速突破，生产力发展正处于从量的积累迈向质的飞跃的关键阶段。面对新形势，国资央企必须着眼开辟增长“第二曲线”，因企制宜、统筹施策，推动新旧动能顺畅有力接续，加快打造一批引领未来竞争的新兴支柱产业，为更好构建以先进制造业为骨干的现代化产业体系提供支撑。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;瑞士全民公投否决“人口上限”倡议&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;瑞士全民公投日前否决了由瑞士人民党提出的“人口上限1000万”倡议，54.79%的选民投下反对票。该提案要求到2050年前将全国常住人口控制在1000万以内，并在达到950万人后启动限制移民措施，必要时终止与欧盟人员自由流动协议。由于其可能冲击瑞士与欧盟的制度性联系，被部分媒体称为“瑞士脱欧”公投。此次投票结果反映出瑞士社会虽然对人口增长、住房紧张、公共服务压力及移民问题存在担忧，但多数选民最终选择优先维护经济利益与对欧关系。作为非欧盟成员国，瑞士长期通过双边协议深度融入欧洲单一市场，其出口超过一半流向欧盟，同时医疗、建筑、酒店、科研等行业高度依赖跨境劳动力。若限制人员自由流动，不仅可能影响劳动力供给，还可能动摇瑞士进入欧洲市场的重要制度基础。从更广泛的欧洲背景看，移民议题仍将持续升温。人口老龄化、劳动力短缺与社会承载能力之间的矛盾不会消失，相关争论未来仍可能以不同形式重新出现。分析认为，对于瑞士而言，这不仅是一次人口政策投票，也是在欧洲政治经济格局变化背景下，对开放发展道路的再次确认。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;美国5月制造业产出行业分化显著&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;美国制造业在连续四个月扩张后，于5月骤然失速。美联储近日公布的数据显示，美国5月工厂产出环比几乎零增长，远低于彭博经济学家调查预期中值0.3%的增幅。此次制造业产出停滞的核心矛盾，在于非耐用品板块受到明显冲击。化工与石油产品产出下滑，合成染料与颜料产出在过去三个月累计下降5.5%，美联储数据显示这可能与战争引发的供应链紊乱有关。与之相对应的是，计算机与电子产品产出在截至5月的三个月内累计增长逾4%，为近五年来最大涨幅，数据中心建设热潮对相关制造业的拉动效应持续释放。国防与航天设备产出连续第六个月攀升，达到2019年12月以来最高水平。经济学家认为，补充战争消耗弹药的需求，以及近期贸易协议框架下出口扩大的潜力，将成为今年制造业增长的重要驱动因素之一。彭博经济学家Stuart Paul表示，数据中心建设与部分回岸投资推动了资本支出计划，耐用品制造为工业产出整体走势提供了支撑，但这远非制造业全面复兴，估计仅约三分之一的品类实现了增长。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;多地高校开展横向科研项目自查自纠工作&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近期国内多所高校陆续启动横向科研项目自查自纠工作。6月11日，海南大学科学技术发展院发布通知，要求对2023年至2025年期间立项、在研、结题的横向科研项目开展自查，重点排查虚设项目、虚增科研体量、经费使用不合规、虚假列支、虚开发票套取科研经费、结题率低、挪用结余经费以及学术不端等问题。此前，湖南省教育厅也已要求省内高校开展近三年横向科研项目全周期自查，长沙理工大学、湖南科技学院、岳阳职业技术学院等高校相继跟进。浙江、河南、山东、广西、内蒙古等地高校也在强化科研经费审计监督，部分学校将自查范围扩大至“十四五”以来纵向、横向及校内科研项目。高校科研经费管理，尤其是横向科研项目，正在成为教育系统审计监督和腐败治理的重要领域。这一轮集中高校自查释放出明确信号：高校科研经费管理，尤其是横向科研项目，正在成为教育系统审计监督和腐败治理的重要领域。横向项目本是高校服务企业、地方和社会需求的重要渠道，也有助于缓解科研经费不足、推动科技成果转化。但从多地自查内容看，横向项目在实际运行中已暴露出一系列共性问题，包括项目真实性不足、经费使用不规范、项目长期停滞、结余资金管理混乱，以及通过中介和企业“配合完成横向课题”的灰色链条。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;美国独立机构之争牵动美联储地位&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近年来，美国最高法院围绕国会设立独立监管机构、总统人事任免权、单一行政权理论等进行了系列庭审辩论。其中，卡瓦诺、阿利托在庭审质询环节辩护指出，国会不能随意增设独立机构插手另一联邦分支事务，二人共同反对民主党设立监督最高法院的独立伦理委员会。分析指出，民主党在国会中推出独立伦理委员会法案本质是借伦理争议设立外部机构约束保守派大法官，削弱特朗普留下的司法长期影响力，而二人公开强硬反对该法案，并从法理层面否定国会干预最高法院伦理监管的权限，守住了司法自主监管的底线，保全了特朗普一手塑造的保守派司法阵地，对特朗普来说也是一次重要的胜利。安邦智库（ANBOUND）首席教授陈功认为，上述言论，对美联储的地位也有部分影响！按照该思路，民主党原本打算推出专门外部机构紧盯美联储政策、人事与经费，以此约束央行决策，但保守派大法官对于国会不能随意增设独立机构插手另一联邦分支事务的言论，会直接给民主党收紧美联储监管的立法设置法律阻碍，保住美联储一定程度自主空间。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;临床科研领域可能成数据安全专项治理重点&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近年来，《网络安全法》《数据安全法》等密集落地，三级医院评审、电子病历分级评价等也陆续将数据安全列为硬性考核指标。今年上半年，多部门强监管的信号密集释放。近日，“严守医疗数据安全”被国家卫健委等14部门列为行业年度反腐纠风工作的独立任务。然而，根据中国医院协会信息专业委员会的调研，医疗机构对相关监管要求的落实工作已取得阶段性进展，但在执行深度与覆盖广度上，仍未达到预期目标。在政策落地“最后一公里”梗阻明显，仅57.5%的医院完成制度修订，32.64%已开展合规建设，近七成医院仍处于“计划中”。在一些数据安全治理的关键环节和关键应对技术投入上，医院仍存在核心能力短板。在与第三方合作中，84.86%的医院与合作对象仅靠保密协议，仅26.11%做数据脱敏，43.19%实现权限闭环；同时重对外防御、轻内部监管，员工违规访问、数据滥用风险突出，进一步加剧三角矛盾。在医学科研个人敏感信息保护中，分别有约六成和五成的医院采取了“设置访问权限”和“签署保密协议”等管理层面的做法。但对于“数字脱敏”“数据匿名化处理”“建设面向临床科研应用的大数据中心”和“数据及时销毁”的核心技术，医院投入占比则分别为33.6%、25.69%、17.92%、12.92%。换言之，在医院数字安全治理中，仍存在一定的“强管理、弱技术”的问题。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;香港收紧劳动力引入政策&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;为缓解当地劳动力不足推出的“补充劳工优化计划”政策推行近三年后，中国香港特区政府于近日宣布了针对该项政策的优化更新措施。根据该计划的最新版本，香港针对外来劳动力（当地称“外劳”）的相关审批政策将增设两级审批机制，并率先在当地的饮食业内推行，包括厨师、初级厨师、烧烤厨师、餐饮调配员及酒吧主管等职位。与相对宽松的第一级审批相比，相关岗位在进入第二级审批机制后，当地劳工与外劳的人手比例，也将由目前的二比一收紧至三比一，即当地雇主至少要聘请三名香港本地员工，才能聘请一名外劳。香港劳工处也强调指出，获得批准输入劳工的雇主，必须与外劳签订标准雇佣合约，并支付不低于同类职位中位工资的薪金。劳工处会维持每月中位工资的规定，并持续优化更新中位工资统计数据的安排，以反映劳动力市场情况。在解释为何首先在餐饮业内引入第二级审批制时，香港劳工处处长许泽森表示，近年来当地结业的餐厅多为中式及大型餐厅，其员工年龄、年资和工资都较高。与此同时，该行内则仍有5%的空缺率和6%的失业率。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;中国有限填补美国留下的全球援助体系“空缺”&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据彭博商业周刊报道，特朗普政府削减数百亿美元美国对外援助后，一些长期依赖美国公共卫生和发展资金的国家出现资金缺口，中国正在尝试以较小规模援助进行有限填补，以此扩大在全球南方国家的影响力。南非抗艾项目是一个典型案例。去年11月，中国驻南非大使在比勒陀利亚宣布，中国将提供350万美元，用于帮助南非防止艾滋病传播。南非约有800万人感染HIV，是全球艾滋病负担最重的国家之一，相关援助具有现实紧迫性。不过，与美国过去的支持规模相比，中国援助仍然有限。此前，美国通过“总统防治艾滋病紧急救援计划”（PEPFAR）每年向南非抗艾工作提供超过4亿美元资金，支持政府宣传、非政府组织、医疗中心和药物治疗，并帮助降低感染率和艾滋病死亡率。特朗普削减对外援助后，这一生命线被压缩，受援国公共卫生体系面临药物供应、基层服务和社会组织运转压力。由此看，中国并非在全面接管美国援助体系，而是在美国退场或收缩后，选择部分高可见度、政治信号强的领域进行补位。这种援助金额虽小，却具有较强象征意义：一方面，它能够凸显中国愿意在公共卫生和发展议题上提供支持，强化在非洲等全球南方国家中的形象；另一方面，也暴露出美国援助政策反复对受援国造成的不确定性，削弱美国长期积累的软实力。总体来看，美国撤出全球援助体系后，确实为中国提供了一定的外交空间。在逆全球化的趋势下，全球多边框架正在遭遇考验，中国也选择了一种更现实的方式应对。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;美国短期内释补战略储油的计划可行性成疑&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据美国能源部6月15日公布的数据，美国战略石油储备（SPR）目前约为3.40亿桶，已降至1983年以来最低水平。不过，就在几天前，特朗普政府还计划从该储备中释放1.72亿桶原油，作为美国与以色列对伊朗发动攻击后全球协调行动的组成部分，旨在抑制因战争推高的油价。若上述计划全部落实，将成为SPR历史上规模第二大的释放行动，储备量将进一步降至约2.43亿桶，仅相当于法定容量的三分之一。此外，能源部表示，计划在未来一年内补充约2亿桶，较本次释放量多出约20%。根据安邦智库（ANBOUND）的研究人员观察，美国这“一释一补”的计划落地可行性成疑。据了解，美国补油来源主要有四类：本土页岩油企业以实物特许权费上缴原油、联邦地块新增开采原油、国际市场采购中东拉美原油、扣押制裁船只原油入库。而现行条件对上述补库方式存在显著制约。一是资金层面国会未足额拨付原油采购预算，全额采购2亿桶原油需巨额财政支出，现有拨款仅能支撑小规模试采购。二是设施层面墨西哥湾沿岸盐穴储库老化，同步释放与入库无法并行，大规模补库需等待本轮1.72亿桶投放全部结束。三是市场层面伊朗冲突持续扰动中东供油通道，国际油价高位震荡，低价囤油窗口期难以稳定出现，OPEC+减产政策也会压缩可采购原油供给。虽然目前地缘层面中东局势暂时缓和，美国逢低采购中东、拉美原油的空间扩大，但在其他三个条件制约下，短期仅能提升海外采购渠道的补货效率与性价比，难以支撑一年内足额完成2亿桶补库目标。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;谨慎看待澳门作为葡语西语联系人的成效&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近日，澳门招商投资促进局行政管理委员会主席谢永强表示，依托“一国两制”下的独特定位，澳门正推动中葡平台功能提质升级并实现战略延伸。一方面，巩固深化中葡传统合作，另一方面，战略延伸至西班牙语国家市场，这是“十五五”期间中葡平台功能的重要突破。此前，澳门经济学会理事长柳智毅曾指出，发挥好“精准联系人”的独特功能，澳门必将在新时代中葡西商贸合作中迎来更大发展机遇，更好助力澳门经济适度多元发展。从战略定位看，澳门打造中葡西合作平台具有一定现实基础。但同时也需要看到，葡语、西语国家的经济重心高度集中于少数大型经济体，且其中不少国家长期处于美国经济、金融和地缘影响范围内。在当前“美洲世纪”背景下，美国持续强化对拉美地区产业链、资源和投资关系的影响，中国企业进一步拓展相关市场可能面临一定外部约束。因此，澳门作为“超级联系人”的实际成效仍需结合国际环境变化进行审慎评估。在此背景下，澳门更好的选择可能是发挥自身特色，成为中国连接葡语国家产业资源的重要节点，发展成为类似“小型产业中介总部”的区域合作平台，并依托粤港澳大湾区产业能力和中国企业资源，连接中国制造、资本与葡语国家资源市场。通过差异化定位，澳门有望在能源、矿产、基础设施、贸易服务等领域形成新的竞争优势，并为自身经济适度多元发展拓展新的增长空间。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;盘谷银行为我国中小银行穿越周期提供选择&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;当前，国内银行业正处在减量提质深度改革周期，中小银行成为行业风险承压最突出板块。2025年全年共计443家中小银行机构通过合并、注销退出法人资质，其中村镇银行276家，退出规模超过前三年总和。全国现存312家高风险银行全部为中小机构，包括14家城商行、191家农信机构、132家村镇银行。截至2026年一季度，商业银行行业平均不良率1.51%，城商行不良率1.85%、农商行不良率2.79%，大幅高于大行1.22%的不良水平。盈利端压力进一步凸显，2026年一季度农商行净利润同比大跌30.24%。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;在安邦智库（ANBOUND）的研究人员看来，这是过去地方中小银行深陷盲目扩规模、扎堆地产与城投信贷、跟风非标投机的历史遗留包袱，在大行下沉、净息差收窄的双重挤压下进退两难。国内中小银行如何告别粗放扩张老路、实现长效稳健经营，泰国盘谷银行陈氏家族三代传承的稳健经营模式，正是可参照的对象。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;在东南亚金融版图上，泰国盘谷银行是一座屹立八十余载的丰碑。陈智深，作为陈氏家族第三代传人、现任盘谷银行总裁，执掌泰国最大商业银行三十余年。在东南亚金融格局剧烈变动、行业争相扩张抢规模、追逐短期高收益的时代浪潮里，他始终不改初心，不追风、不冒进、不赌周期，以“稳健”为核心密码，写就百年银行的发展底色。截至2025年末，盘谷银行总资产达9200亿元人民币，全年净利润104亿元人民币，同比增长8.3%，在泰国银行业中位居前列，继续稳居东南亚第六大商业银行地位。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;陈智深的稳健，源于家族百年传承的商业基因。盘谷银行由其祖父陈弼臣于1944年创立。彼时战火未熄、经济凋敝，陈弼臣以潮汕商人特有的审慎与坚韧，从20万美元起步，打破西方银行垄断，不做投机生意，不碰高风险泡沫，铸就盘谷银行最初的底色。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;父亲陈有汉执掌盘谷银行后，将“稳健”理念推向制度化。他摒弃家族式粗放管理，引入现代金融治理体系，提出“SMILE”五大经验准则，把风险、服务、管理、信贷与人才纳入稳健体系。1983年石油危机冲击泰国，陈有汉敏锐预判风险，果断放慢信贷扩张、归还海外贷款，成功避开经济萧条的冲击。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;陈智深自幼浸润在家族的稳健氛围中，求学于英国名校，系统学习现代金融理论，既懂潮汕商人的“义利并举”，又熟稔西方金融的风险管控逻辑。1994年，他正式接掌盘谷银行。面对外界劝他大举扩张、并购冲刺、做大资产规模的声音，他始终不为所动，而是延续家族“稳扎稳打、步步为营”的传统，将“稳健”作为经营的第一准则。在他看来，盘谷银行不做赌徒银行，不做周期银行，只做世代银行。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;1997年，亚洲金融危机爆发，泰铢大幅贬值、金融体系崩塌，盘谷银行作为泰国最大商业银行，首当其冲陷入绝境。当年纯利润暴跌80%，坏账率飙升至29.8%，资产规模大幅缩水，银行濒临危机边缘。面对危局，陈智深没有慌乱失措，更没有盲目跟风抛售资产、收缩业务，而是以“稳”字当头，制定了一套“止血、固本、重生”的稳健策略。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;他果断出售旗下友联财务公司、曼谷第一信托、亚洲证券公司等非核心资产，快速回笼资金、缓解流动性危机。同时，他积极引入外资、增资扩股，主动降低家族持股比例，从30%降至10%-15%，以开放姿态增强银行资本实力。甚至他亲自坐镇办公室，每天工作至深夜十一二点，逐笔审核坏账、梳理信贷风险，对每一笔业务、每一份报表都审慎核查。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;最终，盘谷银行成功穿越亚洲金融危机的惊涛骇浪。至2000年，盘谷银行逐步恢复盈利，坏账率持续下降，资本充足率稳步回升。这场危机，不仅让盘谷银行站稳脚跟，更让陈智深的稳健经营理念深入人心。在陈智深的带领下，盘谷银行形成了一套独特的稳健经营体系，以风控、服务、布局三大核心，筑牢百年根基。这套体系对症国内中小银行现存弊病，为其未来破局提供参照。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;第一，搭建全方位风控体系，筑牢稳健经营的生命线。风控缺位、资本储备薄弱是国内中小银行最大痛点，过往多数机构为冲业绩放宽授信门槛、大额投向单一高波动行业，一旦行业下行不良集中爆发，资本瞬间被侵蚀。在陈智深的主导下盘谷银行建立了“全流程、全维度”的风控体系。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;一方面，落地信贷实地尽调制度，告别依托抵押物粗放放贷。他坚持“实地调研、审慎评估、从严审批”的原则，要求客户经理深入企业厂房、车间，实地考察生产经营、财务状况。另一方面，持续增厚内源资本，把资本充足率管控摆在经营首位，摆脱过度依赖外部增资续命的困境。截至2025年末，盘谷银行普通股一级资本充足率达16.8%，一级资本充足率17.5%，总资本充足率20.9%，远高于泰国监管要求的12%底线，这是国内中小银行化解存量风险的参考。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;二是复刻微笑服务理念，深耕本土做差异化特色服务。大行持续下沉挤压生存空间、同质化价格战内卷，是中小银行盈利走弱的关键。而陈智深立足本土，延续父亲“微笑服务”的理念，坚守中小客户、经济下行不抽贷断贷的服务路线，是中小银行天然优势所在。未来中小银行需彻底跳出“追大户、跨区域”误区，锚定本土特色产业链、个体工商户，依托地缘、人缘优势做精细化普惠金融。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;同时，借鉴盘谷长效客户维护机制，在实体企业经营承压时合理续贷、纾困帮扶，不靠短期高利率获利，靠长期客户沉淀赚取稳定收益，打造本地化口碑壁垒，走出和大型银行错位竞争的“小而美”路线。截至2025年底，盘谷银行在泰国国内拥有约1180家分行，是泰国分支网络最庞大的银行；在海外设有32家分支机构，业务遍及东亚、东南亚、美国和欧洲，始终保持统一的服务标准，验证了深耕客群的长期价值。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;三是坚持稳中求进步伐，拒绝盲目跨界扩张。过往不少中小银行热衷异地设点、跨界理财、信托等副业，多元化反而拖累主业、滋生风险。而陈智深认为扩张是长跑而非竞速，每一步布局，都要考虑风险、考虑长远、考虑可持续。因此，他始终坚持“立足泰国、深耕东盟、布局全球”的稳健扩张战略，每一步布局都深思熟虑。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;在东南亚，2020年，盘谷银行完成对印尼PermataBank的收购，这是东盟史上规模最大的商业银行并购交易之一。收购前，他带领团队深入调研印尼市场、评估风险、制定整合方案，确保收购后平稳过渡、协同发展。在中国，陈智深更是秉持“稳健为先、长期深耕”的原则，先后在上海、北京、厦门、深圳、重庆设立分行，形成“沿海+内陆”的稳健布局。截至2025年末，盘谷银行（中国）总资产达156.2亿元，实现营业收入4.35亿元，利润总额3520万元，核心一级资本净额52.03亿元，资本充足率高达49.33%，远超监管要求。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;从陈弼臣的白手起家、坚守信誉，到陈有汉的制度革新、审慎扩张，再到陈智深的风控为本、稳中求进，盘谷银行的百年传奇，本质上是一部“稳健”的传承史。陈智深以稳健为舵，在金融浪潮中行稳致远。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;在逆全球化持续深化的背景下，无论金融市场如何风云变幻、经济形势如何起伏跌宕，坚守“稳”字初心，构建全方位风控筑牢、延续微笑服务理念、推进稳中求胜布局，是盘谷银行延续百年的密码，也为中国中小银行走出周期困境提供了选择。总之，大道至简，以稳制胜。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;最终分析结论（Final Analysis Conclusion）：&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;当下国内中小银行深陷规模激进后遗症，风险高企、盈利承压、加速出清，转型破局迫在眉睫。泰国盘谷银行陈智深三代传承的稳健经营理念，为行业提供参考，即构建全方位风控筑牢资本底盘、延续微笑服务理念深耕本土、推进稳中求胜布局拒绝盲目扩张。坚守本源、严控风险、深耕本土，为国内中小银行穿越周期提供了选择。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;美联储可能按兵不动且小幅度缩表&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;当前，美联储正处在一个典型的“观察期”，本月的议息会议大概率仍会选择“按兵不动”，即维持联邦基金利率在3.50%—3.75%区间，而不是急于降息或重新加息。原因也并不复杂，一方面，美国通胀还没有真正回到2%的目标附近，4月PCE同比仍在较高位置，核心通胀黏性也没有完全消除；另一方面，就业市场虽有降温迹象，但失业率仍大致维持在4%左右，并未出现足以迫使美联储快速转向的衰退信号。市场预期也在向这一判断靠拢，最新利率期货显示，6月会议维持利率不变的概率接近九成以上，说明投资者已经基本接受“高利率停留更久”的政策状态。更值得关注的是缩表节奏。美联储6月公布的H.4.1数据显示，截至6月10日，其持有美国国债约4.48万亿美元，MBS约1.96万亿美元，总体资产负债表仍在6万亿美元以上。虽然规模较疫情高峰已有明显下降，但银行体系准备金仍处于相对充裕区间，货币市场运行也较平稳，这给美联储继续小幅度缩表留下空间。也就是说，美联储现在并不急于通过降息释放宽松信号，也没有必要猛烈缩表制造流动性冲击，更可能采取“利率不动、缩表慢走”的组合，即用高利率压住通胀预期，用温和缩表回收过剩流动性，同时避免对美债市场和银行体系造成新的压力。对全球市场而言，这意味着美元利率中枢仍会维持偏高，美债收益率难以快速下行，新兴市场资本流动和汇率压力也不会很快解除。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;日本央行将基准利率上调25个基点&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;6月16日，日本央行宣布将基准利率上调25个基点至1%，达到1995年以来最高水平，并宣布将于2027年4月起暂停缩减国债购买规模。两项决议均以7比1的投票比例通过。此次加息符合市场预期。日本央行在声明中警示，核心CPI通胀率存在向上偏离物价目标的风险，CPI同比涨幅可能加速至明显高于2%的水平，并特别点名油价上涨传导正以＂相对较快的速度＂推进，可能蔓延并推高广泛商品和服务的消费者价格。央行同时表示，将根据经济活动、物价及金融状况的发展，继续提高政策利率。在缩债安排上，央行宣布自2027年4月起将每月国债购买规模维持在约2万亿日元，不再进一步压缩，并取消此前的中期评估惯例。此举意味着央行在维持加息路径的同时，对量化紧缩节奏踩下刹车，在政策取向上形成一定的内部平衡。在日本央行升息后，日经225指数涨超0.5%，触及历史新高；东证指数收复跌幅，转为涨跌持平。西部证券海外分析师张泽恩表示，此次加息属于应对汇率与输入性通胀的被动之举，并非基于经济过热的主动收紧。具体来看，中东地缘局势紧张推升国际油价，显著加剧输入性通胀；日元持续承压贬值，加大进口成本；居民薪资上调幅度超预期，强化工资-物价通胀螺旋；欧洲央行率先加息，外部政策环境形成倒逼。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;外资村镇银行加速退出&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;今年以来已有逾100家村镇银行获批退出。在近期村镇银行改革重组浪潮中，外资机构的持续退出尤为值得关注。近日，汇丰银行宣布北京密云、重庆丰都和湖北麻城三家汇丰村镇银行启动业务转让程序，相关资产、负债及业务将分别移交汇丰中国对应分行承接。加上此前已退出的机构，汇丰在中国设立的12家村镇银行已缩减至7家，县域市场收缩步伐明显加快。近年来，多数外资村镇银行盈利能力持续承压，部分机构长期亏损，导致其资本回报率显著低于财富管理、跨境金融等核心业务板块。值得注意的是，外资银行的退出并不意味着其完全放弃中国市场，而是经营模式正在发生调整。相较于设立独立法人机构深耕县域，未来外资机构更可能将资源集中于跨境金融、供应链金融、财富管理以及数字化金融合作等领域，通过技术和产品输出参与中国金融市场发展。从长期看，外资村镇银行收缩与国内村镇银行整合并行推进，反映出中国县域金融正在从机构数量扩张阶段转向质量提升阶段。未来县域金融体系或将更多依托大型银行分支机构和区域性金融机构构建服务网络，而非依赖数量众多、规模有限的独立村镇银行。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;“新中金”加速成型正式进入监管审批阶段&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;中金公司换股吸收合并东兴、信达证券的汇金系“三合一”重组取得实质推进，该筹划逾半年的重大资产重组申请6月12日获上交所受理并于15日晚间公告，正式迈入监管审核周期。本次交易最早于2025年11月披露，三家机构同属中央汇金体系，中金为A+H头部券商，东兴、信达依托AMC资源深耕本土区域业务，股权架构统一便于整合落地；2025年年末交易预案发布，2026年5月完整草案落地，敲定换股定价与换算比例，中金拟发行31.04亿股A股完成并购，交易完成后汇金仍保持实控地位。以2025年经营数据测算，三方合并后合计营收371.73亿元、归母净利润137.86亿元，年末总资产突破万亿元，一跃成为百亿净利万亿资产级券商。后续项目将先经历上交所多轮问询、重组委审议，通过后递交证监会完成注册，流程走完还需召开三方股东大会履行表决程序，若全部审批落地将启动换股、两家标的摘牌注销、新增股份上市等实施操作。整合落地后，新中金首要任务是推进组织架构、信息系统、营业网点集约化梳理，打通零售客户与机构资源实现交叉销售，放大资本规模拓宽两融、资管、衍生品业务空间，同步强化AMC特色资产证券化业务能力。长期来看，新中金将依托雄厚资本与全渠道布局夯实跨境投行、服务实体产业能力，契合行业打造一流航母级券商导向，但短期层面，也面临人员融合、业务条线梳理、内部同质化业务精简等整合考验，协同红利释放尚需较长周期稳步兑现。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;我国社保资金在期货市场“开户”&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近日，中国期货市场监控中心发文称，近期，用于补充社保基金的国有股权及现金收益类专项养老资产完成首例期货账户开立，可依规开展套期保值业务。本次业务落地，进一步完善了社保基金多层次投资体系，丰富了风险管理工具，助力养老资产有效抵御短期市场波动，实现长期稳健增值，切实守护好百姓的“养老钱”。实际上，长期以来，社保基金等养老资金承担着保障未来养老金支付的重要责任，其在资本市场的参与度越来越高。但随着资本市场波动加剧，尤其是在权益市场波动、利率变化等因素影响下，社保这类长期资金可能面临阶段性净值回撤压力。在此情况下，利用期货市场的风险管理功能开展套期保值就显得尤为重要。金融期货（包括股指期货、国债期货等）能够帮助机构投资者通过对冲工具平滑资产价格波动，从而避免因市场波动被迫调整长期投资策略。从国际经验看，成熟养老基金普遍重视衍生品在资产管理中的作用。养老金投资体系的发展通常经历从保守配置、多元化投资到精细化风险管理的过程。同时，金融期货与现货市场结合，也有助于推动绝对收益、风险平价等投资策略发展，丰富居民财富管理工具。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;各国储备资产配置继续向黄金倾斜&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;世界黄金协会6月16日发布的最新调查显示，全球央行对黄金的配置热情仍在升温。在74名受访储备管理者中，45%表示计划未来12个月继续增持黄金，高于去年的43%；已有黄金储备的央行占比升至93%，也明显高于2025年的81%。这说明黄金已经不只是传统意义上的避险资产，而是越来越多国家重构储备体系的重要工具。过去几年，美元利率高企、地缘冲突频发、金融制裁风险上升，使各国对外汇储备安全性的理解发生变化。相比美元资产，黄金没有发行主体，也不直接依赖某一国家信用，在危机时期更容易被视为“最后的流动性”。尤其是新兴市场和发展中国家，更看重黄金在分散美元风险、对冲通胀和应对地缘政治冲击方面的作用。值得注意的是，央行买金节奏虽可能较2025年放缓约15%，但仍会高于2022年前水平，说明这不是短期投机行为，而是储备资产配置逻辑的中长期调整。同时，部分央行还在提高本土黄金存储比例，反映出对资产可控性和金融安全的重视。总体看，黄金在全球官方储备中的地位正在从补充配置，转变为战略配置，背后折射的是国际货币体系信任结构的变化。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;DeepSeek据悉完成首轮500亿元融资&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;美国科技媒体The Information报道称，中国人工智能初创企业深度求索（DeepSeek）在首轮融资中筹集超过500亿元人民币，企业估值超过500亿美元。据悉，此轮融资采用旨在保留公司创始人控制权的架构。此次融资要求投资者将资金投入由DeepSeek首席执行官梁文锋管理的一家有限合伙企业，而非直接投资于DeepSeek。报道提到，投资者须遵守五年的锁定期安排，且不享有投票权。据The Information报道，中国国家人工智能产业投资基金是唯一的例外。该基金直接投资于DeepSeek，并保留投票权，同时不受五年锁定期限制。路透社本月初报道称，梁文锋已在本轮融资中投入200亿元人民币自有资金。报道也称，中国科技巨头腾讯正考虑投资100亿元人民币，电池巨头宁德时代则考虑投资50亿元人民币，这将使两家公司成为DeepSeek最大的外部投资者。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;英伟达发行250亿美债推动AI算力扩产&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;美东6月15日，英伟达完成250亿美元大额债券发行。本次债券设置2年至30年七档期限，初始募资目标200亿美元，簿记订单峰值达850亿美元，旺盛需求推升发行规模，30年期债券最初给出较美债上浮90个基点的利差指引，最终定价收紧至65个基点，高盛、摩根大通、摩根士丹利联合承销。英伟达2027财年一季报显示，单季经营现金流503.44亿美元，本次发债并非为填补资金缺口。彭博智库分析师Robert Schiffman提出，多期限债券组合可拉长债务久期、锁定偏低融资利率并守住AA级投资评级。英伟达一季报披露新增800亿美元股票回购授权并上调分红，市场普遍认为发债有助于腾挪自有资金投向全球AI算力扩产。据市场统计，2025年五大云厂商发债合计1210亿美元，规模为2020至2024年均值四倍，2026年亚马逊、甲骨文、Alphabet均完成单笔200亿美元以上债券发行。低成本长期资金有望加快公司芯片产能建设与上下游布局，巩固行业资本壁垒。中长期潜在风险仍需警惕，中诚信国际2026年信用周报指出当前科技超长债信用利差处在历史低位；市场普遍预判，若美债长端收益率持续走高将压制存量债估值，全行业加杠杆扩产或放大盈利波动、削弱偿债现金流，信用利差存在阶段性走阔可能。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;资本市场继续支持半导体国产替代融资&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;6月15日，燧原科技和粤芯半导体分别通过上交所科创板、深交所创业板上市委审议，合计拟募资135亿元。两家公司分别对应国产半导体产业链中的AI算力芯片和12英寸晶圆制造环节，均具有较强的国产替代属性。燧原科技成立于2018年3月，总部位于上海临港，主营云端AI芯片及算力系统，是“国产GPU四小龙”之一。公司拟募资60亿元，用于第五代、第六代AI芯片研发及产业化，以及先进人工智能软硬件协同创新项目。腾讯科技是其最大外部股东，与一致行动人合计持股约20.26%，此外还有大基金二期、上海国资等参与。粤芯半导体被称为广州“第一芯”，是广东省自主培养且首家进入量产的12英寸晶圆制造企业。公司拟募资75亿元，用于12英寸模拟特色工艺生产线、特色工艺技术平台研发及补充流动资金。其股东包括广东半导体基金、广州华盈、科学城集团、国投创业基金等。不过，与已实现盈利的长鑫科技相比，燧原科技和粤芯半导体仍处亏损阶段。2023年至2025年，燧原科技净亏损分别为16.65亿元、15.1亿元和11.64亿元，且对腾讯销售占比较高；粤芯半导体近三年累计亏损超过65亿元，预计最早2029年实现盈利。因此，两家公司过会一方面显示资本市场继续支持国产半导体关键环节融资，另一方面也意味着持续亏损、客户集中、供应链稳定和盈利兑现仍是后续观察重点。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;欧洲央行上调今年通胀预期&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;欧洲央行最新上调通胀预期，说明欧元区抗通胀还没有真正结束。根据其最新预测，欧元区2026年总体通胀率预计为3.0%，高于3月预测的2.6%；2027年预计为2.3%，也高于此前2.0%的判断，直到2028年才可能回到2.0%的目标附近。核心通胀同样偏粘性，预计2026年和2027年均为2.5%，2028年仍有2.2%，显示价格压力已不只是能源短期冲击，而是逐步传导到服务、工资和企业成本之中。欧洲央行此次加息25个基点，将存款利率提高至2.25%，正是对通胀回升风险的回应。问题在于，欧元区经济增长并不强，IMF已下调欧元区增长预期，意大利等经济体也面临低增长压力，货币政策因此陷入两难：继续加息有助于压制通胀预期，但会进一步抬高融资成本，压制投资和消费；若过早放松，又可能让通胀重新固化。对欧洲而言，当前真正的风险不是单月物价反弹，而是高能源成本、工资补偿、产业链重构和财政扩张共同推高长期价格中枢。欧央行上调预期，实际上是在提醒市场，欧洲已经很难回到过去低通胀、低利率、低成本的增长环境。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;SpaceX上市后股价快速拉升引估值担忧&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据彭博社6月16日报道，SpaceX日前完成重磅上市后，股价在公开市场继续快速拉升。公司股票在纽约盘前交易中上涨11%，若涨幅延续，将在上市后第三个交易日进一步扩大涨势。此前，SpaceX上市后的前两个交易日累计涨幅已超过40%，这意味着其短短三个交易日内累计涨幅有望超过50%。这一表现显示，公开市场投资者对SpaceX的追捧并未在首日上市后降温，反而继续将其作为稀缺科技资产投资标的进行定价。SpaceX之所以受到资金热捧，一方面在于其长期以来是全球最受关注的非上市科技公司之一，业务横跨火箭发射、Starlink卫星互联网、商业航天和未来太空基础设施；另一方面，随着AI基础设施、低轨卫星通信和太空经济叙事升温，市场也在将SpaceX纳入更广义的科技基础设施平台来估值。对许多投资者而言，SpaceX上市提供了直接参与这一长期成长故事的机会，短期稀缺性和情绪资金共同放大了股价涨幅。不过，快速上涨也带来估值风险。SpaceX虽然拥有较强技术壁垒和商业想象空间，但上市初期股价在三个交易日内可能上涨逾50%，已明显超出传统基本面缓慢验证的节奏，更多体现为市场对未来增长、马斯克影响力和太空经济前景的集中重估。一旦Starlink盈利能力、发射业务现金流、AI或太空基础设施扩张进展不及预期，或市场风险偏好回落，过快拉升的估值可能面临回调压力。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;监管收紧下内地投资者加快锁定“离岸通道”&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据英国《金融时报》6月16日报道，近期中国监管部门加强跨境投资监管后，部分内地投资者反而加快赴港开设银行和投资账户，试图在监管进一步收紧前锁定香港这一“离岸通道”。近期内地处罚了多家被指协助内地客户违规投资境外市场的券商，香港方面也要求券商和银行加强内地客户开户及客户关系审查。这使部分内地投资者担心，未来个人在港开户、购买海外股票、配置美元资产和购买香港保险的便利性可能下降，因此出现“越收紧、越抢先开户”的反应。《金融时报》提到，这一情形与2016年银联收紧内地居民赴港购买保险时相似，政策预期本身会触发投资者提前行动。从资金动机来看，内地投资者并非单纯追逐高风险资产，而是在低利率、资产收益下行和人民币资产配置压力下，寻求美元保单、海外股票和离岸财富管理工具等替代渠道。香港作为内地居民最熟悉、制度距离最近的离岸金融中心，仍具备银行账户、保险、券商、财富管理和美元资产配置的一站式优势。不过，监管收紧也正在改变香港金融机构的经营环境。路透社报道称，中国对跨境投资的整治可能影响香港银行、保险公司和财富管理机构的内地客户业务，AIA、汇丰、保诚、渣打等依赖内地财富流入的机构股价一度承压。金融机构也变得更加谨慎，减少内地客户活动和转介安排。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;商业不动产REITs供给扩容但二级市场整体承压&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近日，首批4只商业不动产REITs全部敲定上市时间，均将于6月18日上市交易，一级市场供给明显提速。最新持有人信息显示，相关产品90%以上份额由机构投资者持有，国新资管、中国保险投资基金等长线资金也出现在持有人名单中。这批产品底层资产位于北京、上海、西安等核心城市，涵盖奥特莱斯、办公楼、商业综合体等业态，预计合计募资规模超过140亿元。Wind数据显示，截至6月12日，即将上市和已申报的商业不动产REITs合计达21只，预计整体募集资金规模超千亿元。与一级市场扩容形成对比的是，REITs二级市场近期整体偏弱。截至6月12日，82只二级市场交易的REITs产品近三月平均下跌5.09%。其中，62只下跌，18只跌幅超过10%，最大跌幅达28.20%；同期仅15只上涨。成交额也从5月下旬逾33亿元回落至上周20.39亿元。资金面方面，主力资金持续净卖出，5月20日所在当周净卖出超过1亿元，与4月22日所在当周逾1亿元净买入形成对比。业内认为，短期压力主要来自商业不动产REITs集中发行带来的资金分流和供给担忧，同时底层资产经营表现分化也影响估值。核心城市优质资产和长线资金参与有助于稳定预期，但办公、商业综合体等业态的出租率、租金和分红稳定性仍是二级市场定价的关键。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;上市公司参设私募股权的三种模式&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;今年以来，众多上市公司宣布出资设立私募股权创投基金。根据WIND统计，截至6月16日，年内已有超50家公司宣布斥资设立私募股权基金。从参设基金的合伙人名单中，除了上市公司、创投等专业投资机构外，还包括地方国资、政府引导基金等。其参设私募股权创投基金的主要模式包括三类。一是“上市公司+PE”并购基金模式：上市公司作为有限合伙人（LP）与专业私募股权机构（GP）共同设立有限合伙制基金，通常出资20%–40%，由PE负责募资、投资与管理，聚焦产业链上下游或战略性标的体外培育，成熟后择机注入上市公司。这是当前最主流、监管相对明确的模式。二是参股设立私募基金管理人（CVC模式）：上市公司以财务或战略投资者身份参股由第三方专业团队设立的私募基金管理人，间接参与基金投资决策；或通过子公司／关联方参与。三是上市公司直接作为LP出资参与第三方设立的私募股权基金：上市公司不参与基金管理，仅以有限合伙人身份认缴出资（常见比例10%–30%），委托持牌私募管理人运作，基金投向泛行业或专项赛道（如科创、新能源），侧重财务回报或产业协同。业内人士表示，上市公司设立私募股权创投基金，通常包含以下几个意图：有的公司是为了打通上下游产业链；有的是为拓展新的产业提前进行布局；当然，还有少数公司只是财务投资。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;分步并购走热小股控盘易损中小股东权益&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近期，A股并购重组市场出现明显结构性变化，一类“分步并购”的新型资本运作模式持续升温。据Wind数据统计，自2025年以来，约十余家上市公司采用该类交易方式，企业从获得控制权到披露资产注入预案，平均用时仅4.6个月，交易落地节奏显著提速。该模式具体分为两个阶段，收购方通过小比例股份协议转让，并辅以表决权委托、一致行动安排等机制，以较低成本取得公司控制权，再在短周期内注入优质资产，实现企业主营业务的快速迭代与整合。多位产业专家表示，该操作方式的兴起，源于近年A股并购监管规则优化，叠加产业资本提升资金使用效率、降低一次性收购压力，让控制权更迭与资产整合得以分步落地。此类并购方式能够帮助上市公司快速补齐产业链短板、优化经营结构。需要正视的是，该模式本身存在天然治理短板，企业容易形成“小股份、大控制权”的股权架构。在此结构下，实控人可依托表决权优势主导资产收购决策，存在推高标的估值、变相输送利益的潜在风险。过快的资产注入节奏，也会压缩企业内部磨合与风险核查周期，极易产生商誉减值、经营不及预期等问题，最终损害中小股东合法权益。当前交易所已依托问询开展穿透式核查，市场预判后续监管或将细化信息披露要求，规范分步并购行为，遏制纯套利式资本运作。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;贝莱德进入定期裁员模式&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;全球最大资产管理公司贝莱德近日启动新一轮裁员，涉及约200名员工，占总员工规模不足1%，覆盖投资、运营、科技及私人融资等多个部门。这已是贝莱德过去18个月内第四次调整人员结构。此前，贝莱德曾于2025年两度裁员，并于2026年初再次削减约250个岗位。公司将相关举措定义为“持续优化组织结构的日常纪律”，反映出大型金融机构正逐步将阶段性裁员转变为常态化效率管理。值得注意的是，此轮调整并非孤立现象，而是全球金融行业组织重构的一部分。摩根大通首席执行官戴蒙近期明确表示，未来将招聘更多AI工程师和技术人才，同时减少传统银行岗位，并已在投资银行业务中大规模部署人工智能工具。美国银行、花旗银行、富国银行等机构也已公开表示，随着AI应用深化，员工总量预计将呈下降趋势。从长期看，金融行业正成为AI重塑白领就业结构的前沿领域。贝莱德连续裁员的意义不仅在于成本控制，更在于显示全球金融机构正从传统的人力密集型模式转向“资本+算力+算法”驱动的新运营模式。未来金融业竞争的关键，或将不再是员工规模，而是AI系统与专业人才协同创造价值的能力。&lt;/p&gt;</t>
   </si>
   <si>
-    <t>参阅信息20260617</t>
-  </si>
-  <si>
     <t>23172</t>
   </si>
   <si>
     <t>&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;国内外重要行业动态&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据新华财经报道，从国家文物局获悉，国家文物局近日印发《国有文物资源数据管理办法》。办法将于2026年11月1日起正式施行。办法明确，国有文物资源数据是指由国有文物管理机构组织的以电子方式对所管理的文物资源信息的记录，包括原始数据、加工后数据、衍生数据；国有文物资源数据属于国家所有，由国有文物管理机构承担具体管理职责。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据新华财经报道，标普全球6日发布的最终数据显示，美国6月制造业和服务业综合景气指数为51.9，高于5月的51.5，但低于52.2的初值。美国6月服务业景气指数为51.2，高于5月的50.7，但低于51.3的初值。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;6月港口货运数据延续景气良性&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;巴克莱数据显示，6月中国港口货物吞吐量维持在约6.8至7.2百万标准箱（mn TEUs）的高位区间，显著高于2024年和2025年同期水平。作为反映外贸活跃度的重要高频指标，这表明当前我国出口物流仍保持较强韧性，海外订单和货物出运需求总体稳定。与此同时，6月制造业PMI中新出口订单分项指数重新回到扩张区间，与港口吞吐量持续高位形成相互印证，意味着当月出口数据有望继续保持较快增长。从结构上看，人工智能基础设施投资、全球补库存需求以及部分企业为应对贸易政策不确定性提前出货，均可能对出口形成支撑。不过，也应看到，高港口吞吐量更多反映的是外需和出口端的景气，并不必然意味着国内需求同步改善。未来若欧美库存周期结束、贸易政策调整或全球经济放缓，出口增长仍可能面临一定压力。整体而言，当前出口仍是支撑中国经济的重要力量，但如何进一步增强内需对经济增长的接续作用，仍将是决定经济修复质量的关键。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;效率层面中美算力差距仍十分悬殊&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据彭博社报道，中国正研究未来五年投入约2万亿元建设全国人工智能数据中心网络，头部互联网企业AI资本开支也将继续增长。不过，从算力效率看，中美之间仍存在明显差距。高盛行业研究的市场摘录显示，国产AI芯片虽然在单位IT功率的初始资本支出上可能比进口芯片低40%至50%，但由于芯片性能密度、能耗、集群互联和软件利用率相对不足，其单位有效算力成本反而可能达到进口方案的2至4倍。在部分实际服务器部署和模型推理场景中，华为昇腾910B、910C的日均Token产出约为英伟达H800的六分之一至三分之一。需要注意的是，上述数据高度依赖模型、精度、集群配置和测试口径，不能简单等同于所有国产芯片的固定性能差距，但其反映出的方向较为清晰：美国仍在高端芯片、先进制程、高带宽存储、集群互联和软件生态方面占据明显优势。当前，中国更多依靠西部低成本电力、大规模基础设施建设、系统集成和算法优化弥补硬件短板，这也意味着完成同等算力任务需要投入更多芯片、电力和数据中心资源。总体来看，中美AI竞争已由模型能力延伸至算力基础设施和资本投入，短期内中国算力建设支出仍将保持高位，但高投入更多体现为追赶成本，而非已经缩小了核心硬件效率差距。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;工业旅游价值在于多元融合发展&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近年来，工业旅游在全国各地蓬勃兴起，在政策加持与消费升级驱动下，工业旅游正从浅层观光，向沉浸式体验、数智化运营、多业态融合等方向转型。近年来，镇海炼化凭借赛博工业风、白鹭生态园等特色景观在网络走红。厂区推出了一体化工业游览路线，邀请游客感受硬核工业与自然生态相融的魅力，如今，已累计接待参观游客超3万人次。山东海阳东方航天港，拥有全球现役唯一的专用海上发射船，打造出“火箭发射观礼”这一独特的文旅IP，让普通观众零距离探访航天发射现场。据行业研究机构预测，未来几年，我国工业旅游将保持年均18%的增速，到2029年，市场规模有望突破3000亿元，发展潜力巨大。但也应看到，当前工业旅游仍存在形式单一、同质化严重、IP辨识度低等现实短板。一些由工业遗存改造的文创产业园，红砖墙、复古铁艺、文创市集几乎成了“标配”。有分析人士认为，问题的根本原因在于对当地工业文化独特价值的深度挖掘不够。虽然我国工业旅游已取得长足进步，但对比全球工业旅游占旅游总收入10%至15%的平均水平，我国不足5%的占比暴露了短板，“流量”可观，但“留量”不足，二次消费空间仍未充分打开。工业和信息化部工业文化发展中心副主任孙星认为，一方面要丰富体验内容，延长游客停留时间；另一方面要打通生产端到消费端的直达链路，扩大销售渠道。在此基础上，还需延伸产业链，做足“工业旅游+”文章，“从门票经济转向综合消费，围绕工业旅游场景发展主题商业、特色市集等多元业态，推动与研学、团建、夜间经济等结合。”&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;社保缴纳联动个税数据征管趋严&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据财新网报道，近期不少企业财务及人力资源部门收到税务部门通知，要求对社保缴费基数与个税工资不匹配的问题开展自查，并及时调整申报、补实缴费基数。按照现行规定，员工上年月平均工资处于当地全口径就业人员平均工资60%至300%之间的，应以实际工资作为社保缴费基数；低于或高于这一范围的，分别按下限和上限缴纳。不过，现实中不少企业长期统一按最低基数缴费，2024年全国人大常委会执法检查报告也指出，按社平工资60%缴费的现象较为普遍。过去，社保少缴漏缴主要依靠职工举报、劳动仲裁以及低比例随机抽查发现，覆盖面有限；当前，随着税务部门掌握个税申报数据，社保征管正由“举报和抽查驱动”转向“数据比对和主动纠偏”。这意味着，企业通过压低缴费基数降低用工成本的空间将明显收窄，劳动密集型企业和中小企业短期内可能面临补缴压力、现金流压力和用工成本上升。不过，从长期看，足额缴纳有助于提高职工养老、医疗等权益保障，也有利于减少企业之间依靠社保少缴形成的不公平竞争。总体来看，社保征管趋严释放出劳动用工合规进一步强化的信号，企业需要尽快重新评估薪酬、社保与用工结构，避免历史欠缴情形演变为更大的合规风险。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;新疆未来更注重培育长期竞争力的产业体系&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;副总理张国清日前在新疆调研中央企业支持新疆产业发展和促进就业工作，先后赴伊犁、昌吉等地考察矿产资源、钢铁冶金、纺织服装、装备制造等行业企业。他强调，中央企业要持续深化拓展与新疆务实合作，结合新疆资源禀赋、产业基础和发展规划，加大重点产业布局，推动发展可持续、就业带动能力强的产业项目落地，支持新疆打造根植性强、稳定性高的支柱产业。同时，加快完善交通、电力、通信、油气和工业用水等基础设施，发挥中央企业和援疆省市国有企业作用，推动产业协同、技能培训、校企合作和订单式培养，以产业发展带动就业扩容增收。此前，副总理丁薛祥也赴新疆调研，强调围绕“五大战略定位”推动新疆高质量发展，显示中央近期持续强化新疆产业发展和战略功能建设。从政策重点来看，此轮部署更加突出产业发展与就业、基础设施和国资布局的协同推进，强调通过制造业集群、资源开发和劳动密集型产业相结合，增强新疆产业发展的稳定性和持续性。这意味着新疆的发展思路正更加注重培育具有长期竞争力的产业体系，而不仅是依靠资源开发或财政投入形成短期增长。从更长期战略看，安邦智库（ANBOUND）认为，西部发展的关键并不仅是沿传统意义上的西部开发逻辑推进产业布局，而是更加重视西部开放，通过向西开放不断增强外循环能力，把新疆建设成为连接中亚、西亚乃至欧洲的重要开放枢纽。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;韩国重启钨矿开采短期难改全球供应格局&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;韩国32年来首次恢复商业化钨矿开采，引发美国、日本等国高度关注。日媒近期称，位于韩国江原道宁越郡的上东钨矿今年3月正式恢复运营，由美国阿尔蒙蒂工业公司开发，预计年产量最高可达4600吨。根据长期协议，初期约一半产量将供应美国，其余将面向韩国、日本及欧洲市场。韩国地方政府表示，未来若产量进一步提升，将考虑向日本出口，并推动建设涵盖选矿、冶炼、加工等环节的本土产业链，力争到2029年前形成较完整的钨加工能力，减少原材料直接出口。日本企业则有望依托自身在钨深加工领域的技术优势，与韩国形成产业合作，拓展非中国来源的供应渠道。钨被广泛应用于切削工具、半导体设备、汽车制造以及导弹、防空系统、航空装备等军工领域，是重要的战略金属。中国作为全球最大的钨生产国，约占全球产量八成，并持续加强战略矿产出口管理，推动国际市场加快寻找替代供应来源。美国近年来也积极推动海外钨矿开发，并扩大战略储备，以增强供应链韧性。有分析指出，上东钨矿恢复生产具有较强的象征意义，但短期内难以根本改变全球钨供应格局。一方面，该矿设计产能与中国整体产量仍存在较大差距；另一方面，钨产业竞争不仅取决于矿山资源，还涉及冶炼、材料加工、高端制造以及供应链配套能力。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;AI需求或令今夏中国电力供应承压加剧&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;德意志银行数据显示，在人工智能基础设施建设的强劲驱动下，中国互联网数据服务领域的电力消耗5月同比激增45.4%，增速较4月的42.8%进一步加快。这种由数据中心需求引致的结构性增长，成为中国5月份整体用电量增速由6.0%升至6.9%的关键动能之一，反映出AI算力投资正逐步成为新的电力需求增长极。与传统制造业或居民用电相比，数据中心具有全年连续运行、负荷集中、制冷需求高等特点，其耗电增长具有较强持续性。国家气候中心预计7月气温将高于常年水平，意味着AI领域持续扩张的高耗电需求将与夏季空调制冷负荷叠加，进一步加大部分地区电网迎峰度夏压力，并对跨区域电力调度、储能配置和电源保障提出更高要求。从长期看，人工智能的发展不仅正在重塑数字经济，也正在重塑能源消费结构，未来电力系统建设将更加注重算力布局与电源建设、电网升级及绿色能源供给的协同匹配，以保障数字经济持续发展与能源安全之间的平衡。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;一个工业县税收与经济活跃度指标的“悖论”&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;在中国各项税收中，增值税是最主要的税收来源，而工业企业又是增值税的纳税大户，这也是各地重视大型工业项目招商的原因之一。疫情前，东部某工业县税收收入约为一年40亿元，税收占一般公共预算收入比重约78%。疫情后，税收收入逐年下行，去年已不足30亿元，五年间减少约10亿元，税收收入占一般公共预算收入比重已降至60%。尽管税收收入有所下降，但当地反映经济活跃度的各项指标并未下降。该负责人发现，工业产值与用电量数据仍在增长，但由于减税降费、部分企业“大拆小”享受税收优惠等因素，导致地方留成税收萎缩，叠加考核机制错位，基层财政腾挪空间极为有限。该负责人提到的拆分问题是很多地区的常见问题，特别是在工业强县。一位税收专家判断，一个工业较发达的县，因拆分可能损失的税收每年可能达亿元。在部分地区，由于多种原因，2026年上半年工业的回暖并未完全形成对财政收入的支撑。除了土地拖累效应外，传统的用电量等数据并不能完全反映工业真实状况。有相关人士在调研中发现，有的地区为了维持用电量数据，让当地经济看起来“健康良性”，会想办法增加某些特定产业的用电量来保持总用电量。也有工业重镇的相关政府人士介绍，其所在地区也出现了工业产值、用电量出现大幅增长，但来自企业端的税收并未明显增长的情况，反而是来自资本市场的个人所得税出现大幅增长。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;越南二季度GDP仍保持高增长&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;越南统计总局数据显示，今年二季度越南实际GDP同比增长8.39%，较一季度7.94%的增速进一步加快；上半年GDP增长8.18%，高于去年同期的7.63%，成为东盟经济增速最高的成员国之一。分行业看，制造业表现最强，增长10.23%，批发零售业、建筑业和电力配电行业分别增长9.67%、9.51%和9.34%。公共投资是支撑增长的重要力量，截至6月25日，2026年公共投资总额达300万亿越南盾，约合115亿美元，计划执行率约30%，较5月底提高8个百分点。胡志明市郊区隆成国际机场、河内五条城市轻轨等大型基建项目正加快推进。外贸方面，二季度出口额增长23%至1436亿美元，其中对美国出口增长约20%；但进口额增长39%至1566亿美元，受原油和石油产品价格上涨影响，贸易出现130亿美元逆差。内需和服务业也保持扩张，含餐饮在内的零售额增长14%至1977万亿越南盾，4月至5月新车销量增长5%，外国游客人数增长18%至549万人次。尽管上半年表现强劲，越南政府设定的全年经济增长目标超过10%，若要完成目标，下半年仍需实现约11.9%的更高增速。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;深圳甲级写字楼空置率暂略下降&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;戴德梁行最新统计数据显示，截至2026年二季度末，深圳市甲级写字楼平均租金进一步降至每月每平方米144.2元，较2025年末累计下降3.4%，而距离十年前已下跌约40%，市场持续走“以价换量”的调整路径。从供应端来看，2026年上半年深圳甲级写字楼新增供应20.1万平方米，全市存量规模随之攀升至928.3万平方米。对比2025年全年71.2万平方米的供应峰值，今年上半年新项目入市节奏明显放缓，短期供给压力有所缓解。但中长期供应压力仍居高不下。据戴德梁行统计，2026年年内仍有94万平方米甲级写字楼待入市，未来五年全市在途供应体量持续高位运行。海量存量叠加持续新增供给，让深圳写字楼市场“价格内卷”成为常态，租金下行趋势延续。持续走低的租金水平，大幅收窄了高低品质写字楼的价差，也意外激活了沉寂已久的置换需求。从需求结构来看，上半年深圳写字楼租赁需求呈现多元复苏态势。其中，企业扩租、新设企业入驻、外地企业入深布局等新增需求，占整体租赁成交面积的37%；原有企业提质搬迁、物业置换的升级需求占比达27%。多元需求集中释放，推动上半年甲级写字楼净吸纳量达到17.5万平方米。叠加部分项目延期入市、短期供应收缩，2026年年中全市写字楼空置率较2025年末下降0.4个百分点至29.1%，成为近年市场难得的阶段性修复信号。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;拉美多国推出对华签证便利化政策&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据巴西《圣保罗页报》7月6日消息，针对7月暑期旅游旺季及下半年市场发展需求，巴西、哥伦比亚等多个拉美国家集中出台对华签证便利化新政，旨在吸引中国高净值游客与跨国商务投资，强化区域发展竞争力。此次政策调整包含多项优化举措，各国通过延长中国公民签证有效期、放宽多次往返入境限制、精简签证申请流程等方式，大幅降低中国人员入境旅游、商务往来的制度门槛。拉美各国此番政策调整，核心依托于中国出境旅游与跨境商务活动持续复苏增长的市场趋势，当地普遍认可中国高消费群体的价值，认为中国游客和投资者能够有效拉动本地旅游、航空、酒店等服务业发展，同时推动跨境经贸合作落地。在全球旅游市场与国际资本竞争日趋激烈的大背景下，此次签证优化是拉美国家主动布局的重要举措，兼具短期增收与长期赋能的双重价值。短期来看，新政能够快速撬动中国出境消费市场，扩大本地旅游营收，激活消费相关产业活力；长远来看，各国希望依托宽松的入境政策，吸纳中国在基础设施、能源、数字经济等重点领域的优质投资，持续扩大外资流入规模，补齐产业发展短板，为区域经济稳定增长注入持续动能，进一步深化中拉文旅与经贸领域的双向合作。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;未成年人社媒禁令成效低于预期&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;2025年底以来，澳大利亚率先通过立法禁止16岁以下未成年人使用社媒，成为全球首个以立法形式限制未成年人社媒使用的国家。此后，马来西亚、印度尼西亚等国家也相继推进各自版本的监管方案。但现实反馈并不乐观。澳大利亚禁令实施半年后，多项公开调查显示，其执行效果远低于预期。清华大学于近日发布了《全球多国未成年人社交媒体管控研究报告》显示，禁令虽使主流社交媒体平台的未成年人账号可见度下降约18个百分点，但约七成原有账号持有者仍保留账号，14—15岁群体的实际合规率只有约27%。另据清华研究团队问卷调研结果，只有19.2%的受访未成年人表示屏幕使用时间因禁令减少。日前，澳大利亚纽卡斯尔大学日发表在《英国医学杂志》的研究也显示，约85%的16岁以下受试者在禁令实施三个月后仍在使用受限制的平台，其中54%—67%使用的是自己的账号。而究其原因，面对禁令，未成年人有不少规避手段，且门槛并不高。清华研究团队的问卷调查结果显示，未成年人使用家长账号、谎报年龄、VPN等方式绕过限制现象普遍，表明年龄门槛未能实质性阻断使用行为。这也就导致了风险并未消失，而是发生了迁移。《报告》显示，禁令实施前后，澳大利亚VPN应用的下载量激增近3倍，Lemon8、Yope等此前并不主流的社交替代应用迅速攀升至澳大利亚App Store生活类排行榜前列，其中Yope的注册用户中约有一半是16岁及以下。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;酒店24小时退房制背后的行业存量竞争困境&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近期重庆、贵阳、西安等多地酒店推出24小时退房制，其背后折射此前安邦智库（ANBOUND）一直追踪的酒店行业存量竞争问题。当前酒店行业存量规模持续扩张，商圈内同类门店高度集聚，硬件设施、配套服务与定价体系趋于同质化，激烈的价格战不断压缩行业利润空间，倒逼酒店跳出低价内卷，依托服务细节打造差异化竞争力，24小时退房制便成为酒店引流塑口碑的重要手段。当下行业进入存量竞争阶段，供给过剩加剧内卷，淡季入住率偏低时，酒店推行该制度能盘活闲置客房、减少空房损失。但受限于存量竞争下的成本与效率平衡难题，该模式尚未实现连锁规模化普及，仅集中在高端行政房型或小众平价门店。行业旺季满房阶段，24小时退房带来的碎片化退房节奏，会打乱保洁集中排班模式，降低客房周转效率，同步推高人力、水电等运营成本。因此多数酒店仅将其作为淡季差异化引流的阶段性手段，而非常态化服务标准。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;非洲多国试图提振炼油产业&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近期，在地缘局势引发全球能源供应链波动的背景下，非洲关于发展本土炼油产业、减少进口依赖的呼声进一步增强。加纳总统马哈马近期宣布，本土开采原油将运往本国的特马炼厂炼制。该炼厂曾长期停工，去年底才逐步复产。加纳是西非产油国之一，但原油主要出口海外，国内汽柴油等长期依赖进口。在西南部非洲，传统产油大国安哥拉也积极建设下游产业。3月，安哥拉卡宾达炼厂正式投产，这是该国50多年来首座新建炼厂。此外，安哥拉新建洛比托炼厂，建成后将成为该国最大炼厂，设计原油加工能力为1000万吨／年。在北非，阿尔及利亚去年底宣布了总投资额高达70亿美元的石化产业扩能计划，其中设计年产能达到500万吨的新建哈西迈萨乌德炼厂将于明年投产；埃及2月批准了2026—2027财年炼厂升级改造计划的有关预算，力推炼油增产，减少进口依赖。不过，非洲炼油产业虽在积极发力，努力提高产能，但随着人口增长和经济发展，各国对成品油的需求也将不断走高，加之产能提升的空间有限。因此，在可预见的未来，非洲炼油产业将出现需求与产能双增、供需缺口长期存在的局面。非洲能源商会更是给出了比较悲观的预测，即到2050年，非洲炼油产品净进口需求将从目前的每日200万桶增至340万桶，增幅高达70%。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;南欧房地产升温正在引发监管警惕&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;7月6日，路透报道称，西班牙和葡萄牙正加强对房地产市场的审视，原因是两国房价快速上涨，并已出现局部过热迹象。不过，监管机构目前并不倾向于立即出手干预，因为当前市场距离上一轮房地产泡沫破裂前的高杠杆状态仍有距离。南欧房价上涨的背后，既有欧洲降息预期、旅游复苏和移民流入带来的需求支撑，也有住房供给不足、短租挤占长期租赁、海外买家涌入等结构性因素。尤其是西班牙、葡萄牙近年成为欧洲乃至全球资本配置房地产的热点地区，高净值人群、远程办公群体和退休移民推高了核心城市和旅游城市房价，也加剧了本地居民的住房负担。此前西班牙曾提出对非欧盟购房者征收最高100%房产税，但相关方案推进并不顺利，说明欧洲国家在抑制投机、保护本地居民和维持投资吸引力之间仍存在政策拉扯。葡萄牙也长期面临租金上涨、黄金签证和旅游短租带来的社会压力。由此看，南欧房地产问题已经不只是资产价格问题，而是旅游经济、人口流动、城市治理和金融稳定交织的结构性矛盾。短期内，监管可能更多采取提高银行审慎要求、限制高风险按揭和加强市场监测等温和手段；但如果房价继续脱离收入增长，住房问题很可能进一步转化为社会和政治压力。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;中国卫星发射领域全球横向对比&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;日前，中国航天科技巨头在文昌航天发射场利用“长征八号A”新型运载火箭，成功将一组全新的商业星座卫星送入预定低轨。此次长征八号A常态化一箭多星组网发射，反映中国低轨互联网星座扩容进入常态化发射。发射频次层面，2026上半年全球轨道发射142次，中国完成43次，占全球三成，总量仅次于美国，但美国仅SpaceX一家年度发射量就远超中国全国总和，猎鹰9号依托成熟助推器回收实现航班化高频发射，火箭复用率超95%，单位发射成本仅为中国商业火箭的三分之一左右。运载工具维度，美国拥有猎鹰9、猎鹰重型、新格伦、星舰多级可回收火箭，星舰近地运力达150吨；中国长征八号A、长征五号等一次性火箭运力稳定，国家队批量一箭多星能力成熟，但轨道级完整回收复用仍处于工程验证阶段，民营液氧甲烷火箭尚未实现规模化复飞，单次发射成本偏高，限制组网速度。此外，目前低轨星座规模差距仍然显著。美国星链在轨超万颗，占据全球七成以上在轨低轨卫星；中国星网、千帆两大星座虽远期申报规划总量充足，但合计在轨不足400颗；欧洲一网星座仅六百多颗在轨，且无自主低成本商业火箭，高度依赖外购发射服务；俄罗斯运力稳定但商业化停滞；印度、日韩仅具备中小型一次性火箭发射能力，无大型低轨星座组网实力。分析认为，由于客观存在技术代差，在可回收火箭产业化、商业化运营效率、低轨星座规模化成型速度等方面，中国与美国存在5至10年的发展差距。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;一个靠信息分析赚钱的投资人&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;在华尔街，聚集着大量高学历、高智商的金融精英，他们几乎7×24小时紧盯各类市场数据——宏观经济数据、企业财务报表、资本市场市盈率、各类技术指标，无所不含。华尔街精英们擅长从最新发布的数据中挖掘关键信号，再通过复杂的排列组合来指引投资方向、获取收益。这是一类高度依赖确定性数据来做判断的人群，不过典型市场中还有“非典型的另一类人”，数量可能不多——他们不靠数字，而是靠分析信息来获取其背后所蕴含的趋势、空间、投资机会等，克里斯·卡米洛就属于后者，而且他做得还不错。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;可以说，卡米洛这个人属于非常不典型的投资人：没有金融科班背景，从未在华尔街大行工作过，甚至不太会读复杂的财务报表。他的投资方式与传统路径截然不同，他将其称之为“社交套利”——就是通过观察社交媒体上的信息来进行趋势总结和判断，并据此发现投资机会，然后在华尔街通过数据分析注意到之前抢先买入。卡米洛通常不看股价走势图，不关心市盈率，也不研究管理团队。他常说的一句话是：“当一个信息已经反映在股价里的时候，再去研究它，已经太晚了。”&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;在一次访谈中，他进一步阐释了自己的投资逻辑：传统投资看重财务、管理团队和估值是否合理，技术分析则依赖价格走势和历史数据，而他的操作方法跟这两样都不沾边，他每天都花费数小时浏览Twitter、TikTok、Reddit等平台的评论区与热搜，观察普通人讨论热点。通过泡在社交媒体上，他希望能够比别人更快地察觉到变化或趋势——包括社会文化的变化、消费行为的变化、产品趋势的变化，甚至政府政策的变化等等，然后把它和一个可以投资的公司连接起来。他管这叫“在信息不对称的时候出手”。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;从信息分析的角度看，卡米洛的投资理念在一定程度上与安邦智库（ANBOUND）在信息分析这一领域的实践有一定的契合度，差别可能就是安邦智库没有将成果直接用于投资行为。安邦智库认为，信息分析并非精确研究，而是一种方向性的前瞻判断，因此尤其适用于趋势预测。就像股市走势的预测，如果透明度高了、数据和资料齐全了、大家想法一致了，那你也无从赚钱了。投资者需要的是尽量早、尽量在大多数人没看明白时就进场——这时候更需要的其实是信息分析，是一个大方向，是尽量比别人看得远、看得早。而卡米洛的投资逻辑恰恰踩中了这点——比别人更早捕捉信息趋势，而不是等到数据公布、所有人都看清确定性之后再行动。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;他很具有代表性的一次交易的灵感来自孩子的玩具。大约在2016年，全世界很多国家和地区的孩子都在家制作“史莱姆”——一种黏糊糊、五彩斑斓的软泥，拿在手里捏着玩。这个现象在社交媒体上飞速蔓延，TikTok和YouTube上挤满了孩子们做史莱姆的视频。卡米洛注意到这是一种潮流，判断这种潮流并非局限于单一地区，而是全球性的普遍热潮。他意识到潮流背后藏有商机，便开始寻找有没有一家纯粹做史莱姆的上市公司，但没找到。进一步研究后，他发现史莱姆的核心原料是白胶，而白胶的主要生产商是埃尔默公司。于是他买入了埃尔默母公司纽威品牌的股票，后来该公司收入增长了50%。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;卡米洛在这笔投资上没赚到太多钱，因为体量有限，但这件事的意义在于：全世界有数千万甚至上亿个家庭都有孩子在玩史莱姆，这些父母每天都能看到满桌子的胶水和颜料，但有多少人能把“孩子在玩史莱姆”和“某家上市公司的股票会上涨”联系起来？而这正是卡米洛把信息转化为投资收益的关键一步——信息本身不值钱，把信息和投资标的连接起来的能力才值钱。这是一种投资哲学，就好比安邦智库所说的，信息都是开源的，如何在开源的信息世界里，通过信息分析的能力，输出有价值的观点并得到验证才是真正的能力。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;卡米洛类似的例子还有很多。疫情期间社交封锁后，人们不能去健身房、不能去办公室，于是纷纷骑自行车。卡米洛观察到这个变化，投资了相关自行车公司。电影《饥饿游戏》上映前，他发现社交媒体上关于该片的讨论热度惊人，于是买入狮门影业股票，影片大卖后股价上涨，他获利退出。还有一种洞洞鞋，华尔街投资者一直认为它只是短暂的潮流、不会持久，但卡米洛观察到年轻人、医护人员、各行各业的人都在穿，明星联名款不断引发话题，他判断这并非一阵风，而是一种文化转变，他基于此买入并最终大赚。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;出于对社交媒体上信息的重视，卡米洛甚至还创办了一家公司，用软件监控社交媒体上特定词汇的出现频率。他说，每当有人问他怎么看市盈率、管理团队或价格走势时，他的回答都一样：“除了我关注的这些信号，我什么都不看。”在他看来，在信息传播速度已被社交媒体彻底改变的时代，传统分析方法已经跟不上节奏。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;作为一个非典型的投资人，卡米洛凭借其独特的信息分析的能力，在投资领域获得了相当不错的回报：从2006年开始，他用8.4万美元起步，到2020年将其变成了4200万美元，期间年复合回报率高达77%。这意味着同期超过86%的美国主动型股票基金经理都没能跑赢他。毫无疑问，在华尔街拥挤的市场中，他是一个成功的投资者！&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;对于普通人而言，华尔街大行的精英们距离太远，而卡米洛的投资哲学似乎更有意义。卡米洛本人也说，普通人在某些方面天生比华尔街有优势。基金经理们每天坐在办公室里看报表、开电话会、读研报，没时间刷短视频、追踪最新网红、观察年轻人中间的流行趋势。而普通人每天都浸在这些信息里——你是新潮流的第一批见证者。你不需要精通金融建模，每一次刷手机、每一次逛商场、每一次观察身边人在做什么，都可能藏着一个投资机会。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;过去，信息自上而下流动，华尔街先知道，再传导给普通人。现在不同了，社交媒体让信息自下而上扩散，普通人在第一线看到变化，而华尔街还在后方看报表。谁先意识到真正的趋势，可能谁就会占得先机。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;说到底，卡米洛本质上其实也只是做了一件事：把观察变成判断，再用判断去进行投资。大多数人在社交媒体上看到趋势，只是消费它——刷过去，笑一笑，然后忘掉。卡米洛看到同样的东西，会追问一句：这个趋势背后，有没有一家公司会因此受益？就是这一问之差，或者说就是这种对待信息的方式，让他在十五年的时间里，把八万多美元变成了四千多万美元。其实，这就是信息分析的价值。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;最终分析结论（Final Analysis Conclusion）：&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;一个公司的股票价格和数据谁都能看到，但真正值钱的，是从海量信息中识别出有效信号的能力，以及比别人快一步的行动力。卡米洛用业绩证明了一件事：在一个信息过载的世界里，最有价值的不是拥有更多信息，而是知道怎么分析信息，并根据这些信息判断出趋势、方向等有价值的东西。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;中国消费意愿疲软的压力依然持续&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;德意志银行（Deutsche Bank）近日公布的调查显示，计划增加可选消费开支的中国消费者比例在2026年第二季度降至46%，为一年来最低水平。与此同时，消费者信心同步走弱，调查中认为自身财务状况有所改善以及预期未来收入增长的受访者比例分别下降6个和2个百分点，反映居民收入预期和消费信心仍待修复。消费意愿减弱意味着居民更加倾向于增加储蓄、压缩非必需支出，服务消费和耐用品消费恢复动能可能进一步放缓。与此同时，国际油价上涨推高出行和物流成本，形成新的输入性价格压力，削弱居民实际购买力。受此影响，航空客运量已出现连续下滑，并进一步向餐饮、住宿、旅游等接触型服务业传导，进一步放大了消费走弱的负面影响。整体来看，当前消费疲弱已不仅是短期情绪波动的体现，更反映出收入预期走弱、成本上升与消费信心不振相互交织的态势。未来消费修复的关键，不仅在于扩大促消费政策力度，更在于稳定居民就业和收入预期，增强家庭部门对未来经济环境的信心，从根本上改善消费内生动力。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;美联储7月加息预期明显下降&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近期，美国市场对美联储7月加息的预期明显降温。直接原因是美国6月就业数据弱于预期，非农就业仅增加5.7万人，低于市场预期的11万人，显示此前偏强的劳动力市场开始降温。与此同时，OPEC+决定8月起继续提高产量目标，布伦特原油回落至每桶72美元附近，能源价格下行也缓解了通胀再度上行的压力。在就业走弱、油价回落的双重影响下，市场认为美联储在7月29日会议上继续按兵不动的概率明显上升，期货市场显示维持利率不变的概率约为78%。这意味着，美联储虽然仍面临通胀高于目标的约束，但短期已不必急于继续加息。对全球市场而言，这一变化有助于缓和美元和美债收益率对新兴市场的压力，也为风险资产提供一定喘息空间。不过，美联储政策并未真正转向宽松，后续仍要看通胀、就业情况和油价是否继续回落。如果美国经济只是温和降温，暂停加息可能延续，但如果通胀黏性重新抬头，或就业数据重新转强，9月以后加息预期仍可能反复。总体看，美联储当前进入的是“观望窗口期”，不是明确的政策转向期。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;黄金ETF首次成为中国规模最大ETF&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;据彭博社7月6日报道，华安易富黄金ETF市值已升至约900亿元人民币，超过华泰柏瑞沪深300ETF的约830亿元，首次成为中国市场规模最大的交易型开放式指数基金。此前，华泰柏瑞沪深300ETF长期是“国家队”稳定A股市场、配置大盘蓝筹的重要工具，其规模被黄金ETF反超，具有较强象征意义。这一变化一方面反映金价上涨和资金持续申购共同推高黄金ETF规模，另一方面也显示投资者风险偏好正在下降，对避险、保值和对冲资产的需求明显增强。值得注意的是，黄金ETF规模上升并不意味着资金完全由股市直接流向黄金，基金规模还受到标的价格上涨影响。不过，沪深300ETF失去“龙头”地位，仍说明此前由政策资金和市场托底预期支撑的宽基ETF优势正在减弱。当前，在经济增长预期偏弱、外部风险上升和股票市场回报不确定性增加的背景下，黄金正由传统避险工具加快转变为居民和机构资产配置中的核心品种。总体来看，黄金ETF登顶不仅是基金规模排名变化，也折射出中国资本市场从追逐权益修复转向重视资产安全的配置逻辑变化。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;深圳龙头市值分化折射产业周期更迭&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;截至6月30日，深圳头部上市主体格局发生显著迭代。年初深圳拥有工业富联、比亚迪、招商银行、中国平安四家万亿市值上市企业，至半年底仅工业富联守住万亿体量，总市值1.43万亿元，比亚迪、招商银行、中国平安市值全部跌破万亿门槛，形成本土龙头“三退一留”的格局。市值格局分化源于各行业基本面周期差异，新能源整车赛道受财税政策节奏扰动明显，2025年末新能源购置税新政提前透支消费需求，制造行业出现阶段性供需错配。零售银行板块，招商银行受全行业息差收窄、居民信贷需求低迷拖累，一季度经营增速弱于国有大行。综合金融龙头中国平安一季度营运利润维持正向增长，但权益市场波动放大投资账面亏损，直接拖累当期净利润。本轮深圳本土龙头市值重构，并非短期资本市场情绪扰动，而是区域传统金融、整车制造与高端先进制造产业景气度切换的直观映射。中长期来看，车企产能释放效率、周期型金融机构经营韧性、保险资管大类资产风控能力，将持续决定本土头部企业估值中枢。行业周期起伏、终端需求波动、权益资产价格震荡，仍是所有企业长期需要应对的常态化经营风险。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;多家银行瞄准算力需求推出AI权益银行卡&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;6月中旬以来，平安银行、招商银行、网商银行瞄准AI爱好者、技术群体、小微商户等，推出AI权益银行卡，持卡人在消费、存款、理财金额达标后，可获算力积分、Token Plan套餐、AI经营工具等福利。据平安银行一位网点工作人员介绍，平安银行“AI智算卡”整合算力聚合付费、基础金融服务、专属算力权益等功能，是平安银行与中国银联、腾讯云联合推出的国内首张面向AI算力个人消费用户的借记卡。“开卡、支付、资产提升达标，均可按规则获取算力积分。”6月25日，针对小微企业“用AI门槛高、运营难、获客难、选址难”等痛点，网商银行联合阿里云、芝麻企业信用、高德等生态伙伴，对“生意金卡”全面升级，推出国内首张面向小微经营者的AI权益卡。博通咨询首席分析师王蓬博认为，“中国有超1亿户个体工商户、超6000万家中小企业。当前AI正成为新的生产工具，但对这些小微经营者来说，要用好AI仍有门槛。”此类银行卡依托智能体持续消耗算力带来稳定复购需求，天然适配消费积分兑换算力额度的闭环模式。王蓬博表示，要实现规模化推广仍有诸多堵点，“比如算力成本动态波动可能导致权益兑付成本不可控；各厂商大模型Token标准不统一，造成权益互通壁垒；算力服务权责划分不清晰可能引发消费者纠纷等。”有业内人士预计，未来银行卡的权益和福利，将告别普惠式大水漫灌，走向分层定制、场景跨界、虚实融合三大方向。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;克服“债性思维”仍是银行系AIC主要挑战&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;自2025年AIC股权投资试点扩围至18个城市以来，AIC股权投资签约意向金额已突破3800亿元。据不完全统计，工银投资、农银投资、中银资产等9家AIC上半年参与的投资基金或项目已超58单，接近2024年全年水平。从半导体到商业航天，从具身智能到低空经济，银行系“长钱”正以前所未有的密度涌入国家战略性新兴产业。资产体量上，头部效应更为明显。截至2025年末，工银投资总资产突破2000亿元大关，达2025.77亿元，同比增长10.16%，稳居行业首位；农银投资总资产1322.77亿元；建信投资总资产1269.8亿元；中银资产总资产960.24亿元；交银投资总资产787.61亿元。从盈利表现看，2025年五家国有行AIC合计净利润达184.36亿元。其中工银投资以52.87亿元净利润领跑，同比增长8.85%；农银投资实现净利润42.95亿元，同比增长9.65%；建信投资实现净利润37.91亿元，同比增长7.36%；中银资产与交银投资则分别实现净利润30.25亿元和20.38亿元。上海金融与发展实验室执行主任董希淼表示，AIC已从最初专注于债转股的专业金融机构，逐步演变为支持科技创新的“长期资本供给者”。然而，银行体系根深蒂固的“债性思维”惯性仍是深层挑战。今年4月，工银投资董事长冯军伏坦言，AIC行业的扩容对整个行业提出了更高要求，特别是资本平衡能力的挑战。虽然单个项目很难保证高比例的成功，但站在国家和公司的立场上，如何确保整体利益，对风险还要有一定的把控。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;县区基金“集约化”的两条路径&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;基于县区财政承压和投资效率偏低等现实问题，监管层正收紧县区政府投资基金设立和财政出资渠道。在此背景下，县区基金正从原有“小而散”的运作模式，转向更高层级统筹和集约化管理。业内认为，县区基金主要有两条转型路径。第一，是将原本用于设立本级基金的资金，转向参与市级或省级统筹母基金。县区仍可作为LP出资，借助更高层级平台的专业投研、项目筛选和资本撬动能力，同时通过返投机制、本地项目推荐权等方式继续服务本地产业招商。相比县区分散设立小基金，省市级平台资金规模更大、专业能力更强，也更适合支持硬科技和长周期产业项目。第二，是将过去依托基金实现的招商让利功能，转化为更加规范的产业政策工具。县区可把原有返投、让利、补贴等安排，梳理为标准化的产业补贴、人才支持、研发奖励和落地扶持政策，通过政策组合拳继续培育本地产业，而不是过度依赖自设基金招商。从行业现状看，县区基金的集约化运作具有现实基础。母基金研究中心数据显示，截至2025年底，全国存续县区基金数量占政府基金总数的44%，但单只平均规模不足市级基金五分之一。长期看，资金向省市级平台集中，有助于提升财政资金使用效率，推动政府投资基金从“分散招商”转向“集约化、专业化、链条化产业投资”。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;年内“摘帽”企业成色受到关注&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;Wind数据显示，今年以来，已有61家A股公司成功撤销退市风险警示或其他风险警示，仅6月以来就有35家公司顺利“摘帽”。大部分公司系借助营业收入指标“过线”而脱险，但此类公司净利润仍处于亏损状态。交易所年报问询对其后续盈利能力、持续经营能力予以重点关注。新业务开展的可持续性、前期“非标”事项影响消除的合理性、相关收入确认方法的合规性等，成为监管部门问询的三大核心问题。川大智胜 2025年新增并表4家子公司贡献营收1.14亿元，助推公司“摘帽”。深交所问询要求说明相关业务是否形成稳定业务模式。星光股份因2025年新增光伏组件类业务受到关注，被要求说明跨行进入光伏领域的原因及竞争优势。此外，前期“非标”事项影响消除的合理性也是问询重点。新潮能源虽已“摘帽”，但上交所仍就其报备的实际运营油井数量与官方渠道数据存在差异的原因展开问询。部分公司还因收入确认方法违规收到警示，如原尚股份因将部分应以净额法核算的收入按总额法核算，导致半年报和三季报多记收入，公司及相关责任人被出具警示函。不少公司“摘帽”后已紧锣密鼓谋求转型。不少公司在“摘帽”后迅速筹划资本运作，或推进控制权变更，或收购资产谋求转型升级。中广天择6月2日“摘帽”后，当月便筹划控制权变更，原控股股东将所持28%股权转让给长沙城发文化旅游集团有限公司，是为优化国有资本布局结构。返利科技6月9日“摘帽”后，公告繁枫智能拟通过股份受让成为新控股股东，市场瞩目新主能否为其带来新动能。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;银行“自营直供”卖房凸显不良资产处置压力&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;中国经营报报道，近日，宁夏银行在京东平台正式上线官方资产店铺，集中展示银川及全区范围内的住宅、商铺、厂房等各类抵债房产，全部房源均为银行产权。这一举措并非孤例，近期多家银行纷纷在电商平台挂牌处置抵债资产，“银行自营直供”处置抵债资产的模式引发市场热议。这种模式体现的是，在房地产深度调整、银行业不良资产供给持续攀升的背景下，从传统的批量转让到如今直面C端购房者，银行在不断探索不良资产处置路径。从更深层次看，银行“自营直供”卖房模式的兴起，折射出当前银行面临的不良资产处置压力在不断加大。国家金融与发展实验室副主任曾刚认为，银行处置不良资产的压力主要来自“增量多、处置难”的双重挤压。一方面，房地产深度调整推升了不良资产供给，房企债务违约集中到期，供给持续增长，银行业处置规模已连续多年创新高，不良处置“大年”仍在延续；另一方面，抵押物尤其是房产大幅贬值，加剧了变现难度。南开大学金融发展研究院院长田利辉认为，当前银行处置不良的压力来自三个维度：一是不良规模攀升且结构向零售集中，处置难度加大；二是批量转让导致价格折损与监管指标压力并存；三是中小银行科技与资本不足，难以高效处置。矛盾焦点在于平衡处置速度、回收价值与合规要求，能力短板制约效能。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;港股将迎来密集限售股解禁周期&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;近期港股迎来密集限售股解禁周期，多家券商提示短期市场供给压力上升。摩根士丹利指出，7月与9月将是解禁高峰期，即使企业基本面未明显恶化，大规模股份释放仍可能对市场流动性形成阶段性扰动，并构成短期估值压制因素。个股层面，AI相关新经济标的解禁尤为集中。智谱约6%股份将结束基石锁定期，稀宇科技与上海天数智芯亦在本周进入解禁窗口，其中稀宇科技解禁比例高达45%，对短期流动性预期影响更为显著。部分标的上市以来涨幅已超过10倍，进一步放大了潜在兑现压力。市场人士认为，港股当前处于高波动、高解禁但弱指数的组合环境中，新增供给冲击与增量资金承接能力之间的平衡将成为短期关键变量。在外部利率预期仍未完全稳定、全球资金风险偏好偏谨慎的背景下，解禁潮可能阶段性放大市场波动，但中期仍取决于盈利兑现与产业景气度能否持续支撑估值结构。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;韩国半导体龙头虹吸致次新股破发加剧&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;2026年韩国IPO市场呈现先热后冷的走势，上半年初期新股挂牌热度攀升，中后期市场情绪快速降温，次新股普遍出现估值回调。今年完成上市的18家企业内，已有14家当前股价跌破发行价。上半年市场投机情绪高涨推升新股发行定价，不少上市标的估值存在明显泡沫，个股挂牌后短期套利资金集中抛售兑现，压低次新股价格。韩国股市增量流动性高度集中在AI、半导体头部权重企业，资金抱团虹吸效应突出，多数新上市、经营模式尚未成熟的中小企业难以获得长期资金承接，进一步拉大个股估值分化。韩国金融行业普遍将一级市场修复预期放在下半年，期待多家大型优质企业、高成长核心资产集中上市提振市场情绪，监管层面也同步落地全新双重上市配套指引，完善本土企业挂牌监管框架。中长期维度，监管制度完善叠加优质IPO标的扩容，具备逐步修复韩国一级市场生态的基础，但资金长期固化抱团半导体龙头、中小新股持续流动性匮乏、外部宏观周期波动等结构性问题难以短期消解。市场后续回暖节奏，仍依赖市场资金分配结构与新股估值定价体系同步回归理性。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;上半年基金新开户数为6年来新高&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;新华财经报道，公募基金正在成为资金入市的重要渠道，越来越多的投资者选择通过场内公募基金把握投资机会。上交所官网数据显示，2026年6月全市场基金新开户数为23.36万户，而2025年6月开户数为20.04万户。2026年上半年基金新开户数合计达183.15万户，为6年来新高，较2025年上半年的150.45万户，同比增长21.73%。在基金新开户数劲增的背后，是新基金发行自4月以来呈现逐月回暖态势：4月成立了165只新基金，发行规模合计为890.94亿元；5月成立了132只新基金，月度发行规模提升至1033.69亿元；6月，无论是新基金成立数量还是发行规模均创年内月度新高。数据显示，6月共成立了208只新基金，发行规模合计达到1205.02亿元。投资者购基热情高涨，多只基金因认购资金超过募集规模上限，启动比例配售。比如，7月4日，国海富兰克林基金发布公告称，富兰克林国海北证50成份指数基金原定募集截止日为7月7日，但截至7月3日已超过募集规模上限，募集截止日提前至7月3日，并对7月3日有效认购申请采用比例配售。7月2日，南方基金公告称，南方中证REITs全收益指数基金提前结募并启动比例配售。谈及对后市的看法，摩根资产管理认为，虽然科技行业的盈利增长具有较高确定性，但在市场处于高位区间时，波动率也有可能持续放大。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;地缘政治与存储供应或制约鸿海下半年业绩&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;在AI服务器需求持续增长带动下，鸿海第二季度业绩继续超出市场预期。公司6月实现营收8217.63亿元新台币，同比增长52.11%，虽然较5月小幅回落4.38%，但仍创历年同期新高。第二季度累计营收达2.51万亿元新台币，同比增长39.83%，环比增长18.02%，高于市场预期的2.37万亿元；上半年累计营收4.64万亿元新台币，同比增长34.99%，同样刷新历史同期纪录。从业务结构看，云端网络产品继续成为增长核心。受益于AI服务器及AI机柜持续放量，相关业务保持四大产品线中最快增长速度，已成为推动公司营收增长的主要引擎。与此同时，消费智能产品、电脑终端产品以及元件与其他业务同比均实现增长，其中消费电子需求改善、新品上市及零部件价格上涨，对整体收入形成一定支撑。不过，从环比表现来看，消费电子和电脑产品拉货节奏有所放缓，AI业务成为支撑整体业绩的决定性力量。展望第三季度，鸿海预计AI机柜产品仍将保持放量增长，下半年ICT产品进入传统旺季，整体营运有望实现同比、环比双增长，AI业务占收入比重预计进一步提升。当前全球大型云服务商资本开支仍维持高位，AI基础设施建设尚未进入放缓阶段，为公司提供了持续订单支撑。不过，鸿海未来仍面临若干制约因素。一方面，AI服务器所需存储芯片等关键零部件供应仍然偏紧，对产能释放形成一定约束；另一方面，全球贸易政策、地缘政治及关税调整仍可能影响供应链布局和客户采购节奏。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;两融扩张需警惕资金过于集中硬科技&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;中证数据显示，2026年上半年，全市场融资融券新开户数达96.06万户，较去年同期61.2万户增长56.96%。其中，6月新开户17.9万户，同比增长76.53%。截至6月末，全市场信用账户总量升至1646.59万户。尽管2月受春节和融资保证金比例上调影响，开户数回落至11.67万户，但3月后整体恢复，5月、6月同比增幅均超过70%，显示投资者参与信用交易的热情持续回升。在开户增长的同时，两融余额也突破关键关口。6月23日，A股两融余额首次突破3万亿元；截至7月2日，两融余额进一步升至3.02万亿元，其中融资余额约3万亿元。相比2014年首次突破1万亿元、2025年8月突破2万亿元，本轮两融扩张节奏明显加快，反映市场回暖后杠杆资金需求持续上升。不过，从账户担保和市值占比等静态指标看，当前两融整体风险尚未接近2015年高峰状态。截至6月30日，全市场信用账户平均维持担保比例为296.44%，明显高于约140%的平仓警戒线，显示整体账户仍有较厚安全垫；两融余额占A股流通市值比重为2.85%，也低于2015年高峰时期的4.27%。值得注意的是本轮两融增量资金高度集中于硬科技赛道。短期看，这有助于强化科技主线和市场风险偏好，但相关板块估值快速抬升、交易拥挤加剧，一旦行情反转，杠杆资金集中持仓可能放大局部波动。因此，结构性杠杆和硬科技赛道集中度风险仍需关注。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;美国能源结构的天然气支柱加速强化&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;彭博社近期表示，根据美国能源信息署（EIA）的数据，美国天然气消费量正迅速接近石油，预计到2030年将首次超过石油，成为美国最主要的能源来源。这一结构性转变主要得益于页岩气革命带来的丰富且低成本的天然气供应，其不仅在发电领域大规模替代煤炭，也持续支撑数据中心建设、电动汽车普及等带来的新增电力需求，成为美国人工智能和先进制造业发展的重要能源基础。天然气占比持续提升，意味着美国能源体系正由传统石油主导逐步转向以天然气和电力为核心的新格局，有助于增强能源安全、降低发电成本，并提升产业竞争力。对中国而言，这一趋势既体现了稳定、低成本能源供给对新兴产业发展的重要支撑，也进一步凸显加快构建多元化能源体系的必要性。近年来，中国在风电、光伏、核电、特高压、新型储能等领域已形成较强产业优势，随着深地热、先进核能、天然气调峰和智能电网等基础设施持续完善，中国有望依托多元能源协同和清洁能源规模优势，为人工智能、先进制造等战略性产业提供更加稳定、高效的能源保障，不断增强经济发展的内生动力和国际竞争力。&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;&lt;strong&gt;穆迪预判亚太私募信贷募资投资增速放缓&lt;/strong&gt;&lt;/p&gt;&lt;p style="text-align: justify; text-indent: 2em;"&gt;7月6日，国际评级机构穆迪发布亚太私募信贷市场展望报告，预判未来12至18个月，亚太区域私募信贷募资、投资增速将逐步放缓。全球经济前景不确定性上升、地缘摩擦持续、市场利率维持高位运行，多重约束叠加，降低机构对私募信贷这类低流动性资产的配置意愿。放眼全球市场，海外主流私募信贷基金普遍遭遇集中赎回，倒逼全市场收紧信贷基金流动性条款审核标准。该流动性收紧趋势正向亚太传导，直接制约市场增量资金入场，零售、财富管理渠道受冲击最为突出。资金供给收缩背景下，亚太私募信贷投放节奏、项目风控标准将同步收紧，中小融资主体、非标信贷项目融资落地难度抬升，市场资金进一步向资质稳健、规模较大的头部项目倾斜。中长期来看，亚太私募信贷行业将承受结构性压力，高利率环境将压缩信贷资产收益，区域各国经济复苏分化加大底层资产信用波动，流动性监管完善、基金条款标准化抬高行业准入门槛。综合来看，行业粗放扩张周期宣告收尾，后续将步入增速下行、风控标准升级、资金结构持续优化的调整阶段。&lt;/p&gt;</t>
-  </si>
-  <si>
-    <t>参阅信息20260707</t>
   </si>
   <si>
     <t>TEST_20260826</t>
@@ -80,7 +74,15 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>参阅信息2026-08-27</t>
+    <t>参阅信息2026-08-28</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>参阅信息20260829</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>参阅信息20260830</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -396,7 +398,7 @@
         <v>8</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.15">
@@ -412,16 +414,16 @@
       <c r="D3" t="s">
         <v>8</v>
       </c>
-      <c r="E3" t="s">
-        <v>12</v>
+      <c r="E3" s="2" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
@@ -429,19 +431,19 @@
       <c r="D4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" t="s">
-        <v>15</v>
+      <c r="E4" s="2" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.15">
       <c r="A5" t="s">
+        <v>14</v>
+      </c>
+      <c r="B5" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B5" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="C5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D5" t="s">
         <v>8</v>

</xml_diff>